<commit_message>
Tag the six women who lacked the נשים tag
610 the Rebbetzin Chaya Mushka Schneerson, 611 Geula Cohen, 613 Leah, 614 Sol
Hachuel, 624 Imma Shalom and 629 Miriam lacked the whole tag נשים (Imma
Shalom had only "נשים בתלמוד", and the site matches the whole tag), so the
tower, the Six Steps captions and the description links spoke of them as men
("בן משפחתו של משה רבנו" for Miriam). The tag is appended in the spreadsheet
(six cells, nothing else in the file rewritten) and in both data.json copies
(six nodes, still byte-identical). WOMEN_UNTAGGED is gone from the description
links generator, which now reads the tag alone; the links were regenerated.
Tests pin the six by name in the tower, connect and description-links suites,
and a guard in the terms suite fails when a tag holds the word נשים inside a
longer tag without the whole tag.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SBYugGL8CAuCXRwwBSSyDg
</commit_message>
<xml_diff>
--- a/data/description-links.xlsx
+++ b/data/description-links.xlsx
@@ -556,7 +556,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>1258</v>
+        <v>1261</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -766,7 +766,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="n">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
@@ -2320,40 +2320,40 @@
         <v>43</v>
       </c>
       <c r="B44" s="3" t="n">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>רבנו בחיי אבן פקודה – חובות הלבבות</t>
+          <t>מר שושני</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>«Ховот ха-Левавот»: сущность иудейской этики</t>
+          <t>The Riddle of the Mysterious Genius: Mr. Shushani</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/eEk1_6ItRcY/edit</t>
+          <t>https://studio.youtube.com/video/unqH7pHySmM/edit</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабейну Бахья ибн Пакуда («Обязанности сердец») в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/39?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Mr. Shoshani on Ozar Chachamim — the full research and his teachers and students: https://ozar-chachamim-app.vercel.app/en/sage/148?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/eEk1_6ItRcY</t>
+          <t>https://youtu.be/unqH7pHySmM</t>
         </is>
       </c>
       <c r="I44" s="2" t="n">
-        <v>481</v>
+        <v>699</v>
       </c>
       <c r="J44" s="2" t="n"/>
     </row>
@@ -2366,36 +2366,36 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>מר שושני</t>
+          <t>רבנו בחיי אבן פקודה – חובות הלבבות</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>The Riddle of the Mysterious Genius: Mr. Shushani</t>
+          <t>«Ховот ха-Левавот»: сущность иудейской этики</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/unqH7pHySmM/edit</t>
+          <t>https://studio.youtube.com/video/eEk1_6ItRcY/edit</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>📜 Mr. Shoshani on Ozar Chachamim — the full research and his teachers and students: https://ozar-chachamim-app.vercel.app/en/sage/148?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабейну Бахья ибн Пакуда («Обязанности сердец») в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/39?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/unqH7pHySmM</t>
+          <t>https://youtu.be/eEk1_6ItRcY</t>
         </is>
       </c>
       <c r="I45" s="2" t="n">
-        <v>699</v>
+        <v>481</v>
       </c>
       <c r="J45" s="2" t="n"/>
     </row>
@@ -2618,36 +2618,36 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>הרב יוסף דוב הלוי סולובייצ׳יק (הגרי״ד)</t>
+          <t>רבי שמואל די אוזידא (בעל מדרש שמואל)</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Joseph Dov Soloveitchik - The Halakhic Man Who Lived Between Two Worlds</t>
+          <t>Рабби Шмуэль де Узеда - каббалист из Цфата, спасший мудрость ранних мудрецов от забвения</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/OXMfO24yAeU/edit</t>
+          <t>https://studio.youtube.com/video/KTKuiDElfCY/edit</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Yosef Dov HaLevi Soloveitchik (the Rav) on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/608?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Шмуэль де Узеда («Мидраш Шмуэль») в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/631?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/OXMfO24yAeU</t>
+          <t>https://youtu.be/KTKuiDElfCY</t>
         </is>
       </c>
       <c r="I51" s="2" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="J51" s="2" t="n"/>
     </row>
@@ -2656,40 +2656,40 @@
         <v>51</v>
       </c>
       <c r="B52" s="3" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>רבי שמואל די אוזידא (בעל מדרש שמואל)</t>
+          <t>הרב יוסף דוב הלוי סולובייצ׳יק (הגרי״ד)</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>Рабби Шмуэль де Узеда - каббалист из Цфата, спасший мудрость ранних мудрецов от забвения</t>
+          <t>Rabbi Joseph Dov Soloveitchik - The Halakhic Man Who Lived Between Two Worlds</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/KTKuiDElfCY/edit</t>
+          <t>https://studio.youtube.com/video/OXMfO24yAeU/edit</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Шмуэль де Узеда («Мидраш Шмуэль») в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/631?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Yosef Dov HaLevi Soloveitchik (the Rav) on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/608?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/KTKuiDElfCY</t>
+          <t>https://youtu.be/OXMfO24yAeU</t>
         </is>
       </c>
       <c r="I52" s="2" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="J52" s="2" t="n"/>
     </row>
@@ -3202,7 +3202,7 @@
         <v>64</v>
       </c>
       <c r="B65" s="3" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
@@ -3211,31 +3211,31 @@
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>רבי אלכסנדרי זוסלין הכהן (המהרא״ך)</t>
+          <t>עמנואל לוינס</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>Рабби Александри Зусслин ха-Коэн — законоучитель, сохранивший Тору из пепла</t>
+          <t>Эммануэль Левинас: этика, феноменология и лицо Другого</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/D03fiiP5cJM/edit</t>
+          <t>https://studio.youtube.com/video/vyuGrknqd9g/edit</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Александри Зуслин ха-Коэн (Махарах) в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/319?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Эммануэль Левинас в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/151?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/D03fiiP5cJM</t>
+          <t>https://youtu.be/vyuGrknqd9g</t>
         </is>
       </c>
       <c r="I65" s="2" t="n">
-        <v>213</v>
+        <v>384</v>
       </c>
       <c r="J65" s="2" t="n"/>
     </row>
@@ -3253,31 +3253,31 @@
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>עמנואל לוינס</t>
+          <t>רבי אלכסנדרי זוסלין הכהן (המהרא״ך)</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>Эммануэль Левинас: этика, феноменология и лицо Другого</t>
+          <t>Рабби Александри Зусслин ха-Коэн — законоучитель, сохранивший Тору из пепла</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/vyuGrknqd9g/edit</t>
+          <t>https://studio.youtube.com/video/D03fiiP5cJM/edit</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>📜 Эммануэль Левинас в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/151?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Александри Зуслин ха-Коэн (Махарах) в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/319?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/vyuGrknqd9g</t>
+          <t>https://youtu.be/D03fiiP5cJM</t>
         </is>
       </c>
       <c r="I66" s="2" t="n">
-        <v>384</v>
+        <v>213</v>
       </c>
       <c r="J66" s="2" t="n"/>
     </row>
@@ -3505,31 +3505,31 @@
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>הרב מאיר כהנא</t>
+          <t>עמנואל לוינס</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Meir Kahane – The Ideology, Activism, and Legacy That Continue to Shake Israel</t>
+          <t>Emmanuel Levinas: Ethics, Phenomenology, and the Face of the Other</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/x_YuhpmskCM/edit</t>
+          <t>https://studio.youtube.com/video/e9KpVSP9s9E/edit</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Meir Kahane on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/197?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Emmanuel Levinas on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/151?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/x_YuhpmskCM</t>
+          <t>https://youtu.be/e9KpVSP9s9E</t>
         </is>
       </c>
       <c r="I72" s="2" t="n">
-        <v>564</v>
+        <v>385</v>
       </c>
       <c r="J72" s="2" t="n"/>
     </row>
@@ -3547,31 +3547,31 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>הרב בן־ציון מאיר חי עוזיאל</t>
+          <t>הרב מאיר כהנא</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Ben-Zion Meir Hai Uziel: Thought, Halakha, and Zionism</t>
+          <t>Rabbi Meir Kahane – The Ideology, Activism, and Legacy That Continue to Shake Israel</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/L2hQKYIBlmE/edit</t>
+          <t>https://studio.youtube.com/video/x_YuhpmskCM/edit</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Ben-Zion Meir Chai Uziel on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/138?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Meir Kahane on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/197?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/L2hQKYIBlmE</t>
+          <t>https://youtu.be/x_YuhpmskCM</t>
         </is>
       </c>
       <c r="I73" s="2" t="n">
-        <v>624</v>
+        <v>564</v>
       </c>
       <c r="J73" s="2" t="n"/>
     </row>
@@ -3580,7 +3580,7 @@
         <v>73</v>
       </c>
       <c r="B74" s="3" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
@@ -3589,31 +3589,31 @@
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>עמנואל לוינס</t>
+          <t>הרב בן־ציון מאיר חי עוזיאל</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>Emmanuel Levinas: Ethics, Phenomenology, and the Face of the Other</t>
+          <t>Rabbi Ben-Zion Meir Hai Uziel: Thought, Halakha, and Zionism</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/e9KpVSP9s9E/edit</t>
+          <t>https://studio.youtube.com/video/L2hQKYIBlmE/edit</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>📜 Emmanuel Levinas on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/151?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Ben-Zion Meir Chai Uziel on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/138?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/e9KpVSP9s9E</t>
+          <t>https://youtu.be/L2hQKYIBlmE</t>
         </is>
       </c>
       <c r="I74" s="2" t="n">
-        <v>385</v>
+        <v>624</v>
       </c>
       <c r="J74" s="2" t="n"/>
     </row>
@@ -4462,40 +4462,40 @@
         <v>94</v>
       </c>
       <c r="B95" s="3" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>המהרש״א</t>
+          <t>חכם ציון חביב ברכה</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>Маарша — человек, соединивший разум, сердце и общественную ответственность</t>
+          <t>Rabbi Zion Haviv Bracha – the hidden kabbalist who bridged the generations of the Rashash tradition</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/oKZzcHz2jlE/edit</t>
+          <t>https://studio.youtube.com/video/uS2JTq4xVJo/edit</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>📜 Махарша в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/329?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Chacham Tzion Chaviv Bracha on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/180?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/oKZzcHz2jlE</t>
+          <t>https://youtu.be/uS2JTq4xVJo</t>
         </is>
       </c>
       <c r="I95" s="2" t="n">
-        <v>329</v>
+        <v>560</v>
       </c>
       <c r="J95" s="2" t="n"/>
     </row>
@@ -4513,31 +4513,31 @@
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>רבי יצחק מווינה (בעל האור זרוע)</t>
+          <t>המהרש״א</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>Рабби Ицхак из Вены, автор «Ор Зару́а» — человек, посеявший свет между Талмудами</t>
+          <t>Маарша — человек, соединивший разум, сердце и общественную ответственность</t>
         </is>
       </c>
       <c r="F96" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/ARiH1Rj5xY8/edit</t>
+          <t>https://studio.youtube.com/video/oKZzcHz2jlE/edit</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Ицхак из Вены (Ор Заруа) в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/43?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Махарша в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/329?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/ARiH1Rj5xY8</t>
+          <t>https://youtu.be/oKZzcHz2jlE</t>
         </is>
       </c>
       <c r="I96" s="2" t="n">
-        <v>394</v>
+        <v>329</v>
       </c>
       <c r="J96" s="2" t="n"/>
     </row>
@@ -4550,36 +4550,36 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>חכם ציון חביב ברכה</t>
+          <t>רבי יצחק מווינה (בעל האור זרוע)</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Zion Haviv Bracha – the hidden kabbalist who bridged the generations of the Rashash tradition</t>
+          <t>Рабби Ицхак из Вены, автор «Ор Зару́а» — человек, посеявший свет между Талмудами</t>
         </is>
       </c>
       <c r="F97" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/uS2JTq4xVJo/edit</t>
+          <t>https://studio.youtube.com/video/ARiH1Rj5xY8/edit</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>📜 Chacham Tzion Chaviv Bracha on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/180?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Ицхак из Вены (Ор Заруа) в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/43?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/uS2JTq4xVJo</t>
+          <t>https://youtu.be/ARiH1Rj5xY8</t>
         </is>
       </c>
       <c r="I97" s="2" t="n">
-        <v>560</v>
+        <v>394</v>
       </c>
       <c r="J97" s="2" t="n"/>
     </row>
@@ -6058,40 +6058,40 @@
         <v>132</v>
       </c>
       <c r="B133" s="3" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>רבי חנינא בר פפא</t>
+          <t>פרנץ רוזנצווייג – הפילוסוף שהחזיר את האדם למרכז</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>Рабби Ханина бар Папа - аморай, попросивший у Ангела смерти ещё 30 дней</t>
+          <t>Franz Rosenzweig and His Thought: Jewish Theology and Philosophy</t>
         </is>
       </c>
       <c r="F133" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/oZif-VqdVNU/edit</t>
+          <t>https://studio.youtube.com/video/-KEL3MtX4nU/edit</t>
         </is>
       </c>
       <c r="G133" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Ханина бар Папа в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/543?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Franz Rosenzweig on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/141?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H133" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/oZif-VqdVNU</t>
+          <t>https://youtu.be/-KEL3MtX4nU</t>
         </is>
       </c>
       <c r="I133" s="2" t="n">
-        <v>47</v>
+        <v>478</v>
       </c>
       <c r="J133" s="2" t="n"/>
     </row>
@@ -6104,36 +6104,36 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>רבי דוד הלוי סגל (הט"ז)</t>
+          <t>רבי חנינא בר פפא</t>
         </is>
       </c>
       <c r="E134" s="7" t="inlineStr">
         <is>
-          <t>Rabbi David HaLevi Segal – The Taz: A Halakhic Authority Who Turned Law into Living Reality</t>
+          <t>Рабби Ханина бар Папа - аморай, попросивший у Ангела смерти ещё 30 дней</t>
         </is>
       </c>
       <c r="F134" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/EfMLCZVUz68/edit</t>
+          <t>https://studio.youtube.com/video/oZif-VqdVNU/edit</t>
         </is>
       </c>
       <c r="G134" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi David HaLevi Segal (the Taz) on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/79?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Ханина бар Папа в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/543?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H134" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/EfMLCZVUz68</t>
+          <t>https://youtu.be/oZif-VqdVNU</t>
         </is>
       </c>
       <c r="I134" s="2" t="n">
-        <v>428</v>
+        <v>47</v>
       </c>
       <c r="J134" s="2" t="n"/>
     </row>
@@ -6142,40 +6142,40 @@
         <v>134</v>
       </c>
       <c r="B135" s="3" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>רב האי גאון</t>
+          <t>רבי דוד הלוי סגל (הט"ז)</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>Рабби Хай Гаон – последний из Гаонов и первый из Великих:человек, восстановивший твёрдость Галахи</t>
+          <t>Rabbi David HaLevi Segal – The Taz: A Halakhic Authority Who Turned Law into Living Reality</t>
         </is>
       </c>
       <c r="F135" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/95zK1eE05_w/edit</t>
+          <t>https://studio.youtube.com/video/EfMLCZVUz68/edit</t>
         </is>
       </c>
       <c r="G135" s="7" t="inlineStr">
         <is>
-          <t>📜 Рав Хай Гаон в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/25?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi David HaLevi Segal (the Taz) on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/79?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H135" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/95zK1eE05_w</t>
+          <t>https://youtu.be/EfMLCZVUz68</t>
         </is>
       </c>
       <c r="I135" s="2" t="n">
-        <v>584</v>
+        <v>428</v>
       </c>
       <c r="J135" s="2" t="n"/>
     </row>
@@ -6184,40 +6184,40 @@
         <v>135</v>
       </c>
       <c r="B136" s="3" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
         <is>
-          <t>שלמה מולכו</t>
+          <t>רב האי גאון</t>
         </is>
       </c>
       <c r="E136" s="7" t="inlineStr">
         <is>
-          <t>Shlomo Molcho: The Messianic Kabbalist and His Self-Sacrifice for the Sanctification of God’s Name</t>
+          <t>Рабби Хай Гаон – последний из Гаонов и первый из Великих:человек, восстановивший твёрдость Галахи</t>
         </is>
       </c>
       <c r="F136" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/s7NQCbMVv90/edit</t>
+          <t>https://studio.youtube.com/video/95zK1eE05_w/edit</t>
         </is>
       </c>
       <c r="G136" s="7" t="inlineStr">
         <is>
-          <t>📜 Shlomo Molcho on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/326?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рав Хай Гаон в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/25?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H136" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/s7NQCbMVv90</t>
+          <t>https://youtu.be/95zK1eE05_w</t>
         </is>
       </c>
       <c r="I136" s="2" t="n">
-        <v>334</v>
+        <v>584</v>
       </c>
       <c r="J136" s="2" t="n"/>
     </row>
@@ -6230,36 +6230,36 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
         <is>
-          <t>הרב שמואל מוהליבר – מנהיג דתי ומבשר הציונות</t>
+          <t>שלמה מולכו</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>Раввин Шмуэль Моаливер: пионер религиозного сионизма</t>
+          <t>Shlomo Molcho: The Messianic Kabbalist and His Self-Sacrifice for the Sanctification of God’s Name</t>
         </is>
       </c>
       <c r="F137" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/vUjK21VU1Ww/edit</t>
+          <t>https://studio.youtube.com/video/s7NQCbMVv90/edit</t>
         </is>
       </c>
       <c r="G137" s="7" t="inlineStr">
         <is>
-          <t>📜 Рав Шмуэль Мохливер в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/120?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Shlomo Molcho on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/326?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H137" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/vUjK21VU1Ww</t>
+          <t>https://youtu.be/s7NQCbMVv90</t>
         </is>
       </c>
       <c r="I137" s="2" t="n">
-        <v>472</v>
+        <v>334</v>
       </c>
       <c r="J137" s="2" t="n"/>
     </row>
@@ -6272,36 +6272,36 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D138" s="4" t="inlineStr">
         <is>
-          <t>פרנץ רוזנצווייג – הפילוסוף שהחזיר את האדם למרכז</t>
+          <t>הרב שמואל מוהליבר – מנהיג דתי ומבשר הציונות</t>
         </is>
       </c>
       <c r="E138" s="7" t="inlineStr">
         <is>
-          <t>Franz Rosenzweig and His Thought: Jewish Theology and Philosophy</t>
+          <t>Раввин Шмуэль Моаливер: пионер религиозного сионизма</t>
         </is>
       </c>
       <c r="F138" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/-KEL3MtX4nU/edit</t>
+          <t>https://studio.youtube.com/video/vUjK21VU1Ww/edit</t>
         </is>
       </c>
       <c r="G138" s="7" t="inlineStr">
         <is>
-          <t>📜 Franz Rosenzweig on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/141?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рав Шмуэль Мохливер в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/120?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H138" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/-KEL3MtX4nU</t>
+          <t>https://youtu.be/vUjK21VU1Ww</t>
         </is>
       </c>
       <c r="I138" s="2" t="n">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="J138" s="2" t="n"/>
     </row>
@@ -6352,7 +6352,7 @@
         <v>139</v>
       </c>
       <c r="B140" s="3" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
@@ -8162,36 +8162,36 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D183" s="4" t="inlineStr">
         <is>
-          <t>תודוס איש רומי</t>
+          <t>רבי אלעזר מגרמייזא (בעל הרוקח)</t>
         </is>
       </c>
       <c r="E183" s="7" t="inlineStr">
         <is>
-          <t>Религиозная власть и имперская политика в Древнем Риме</t>
+          <t>Rabbi Eleazar of Worms and the Ordinances of ShUM</t>
         </is>
       </c>
       <c r="F183" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/LJjUME0eG6g/edit</t>
+          <t>https://studio.youtube.com/video/XewrhViUp7E/edit</t>
         </is>
       </c>
       <c r="G183" s="7" t="inlineStr">
         <is>
-          <t>📜 Теодос из Рима в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/485?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Elazar of Worms (the Rokeach) on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/280?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H183" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/LJjUME0eG6g</t>
+          <t>https://youtu.be/XewrhViUp7E</t>
         </is>
       </c>
       <c r="I183" s="2" t="n">
-        <v>458</v>
+        <v>264</v>
       </c>
       <c r="J183" s="2" t="n"/>
     </row>
@@ -8204,36 +8204,36 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>עברית</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D184" s="4" t="inlineStr">
         <is>
-          <t>הרב יצחק יעקב ריינס</t>
-        </is>
-      </c>
-      <c r="E184" s="5" t="inlineStr">
-        <is>
-          <t>הרב יצחק יעקב ריינס ומייסד המזרחי</t>
+          <t>תודוס איש רומי</t>
+        </is>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>Религиозная власть и имперская политика в Древнем Риме</t>
         </is>
       </c>
       <c r="F184" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/BVYplCpF02c/edit</t>
-        </is>
-      </c>
-      <c r="G184" s="5" t="inlineStr">
-        <is>
-          <t>📜 הרב יצחק יעקב ריינס באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/489?utm_source=youtube&amp;utm_medium=video</t>
+          <t>https://studio.youtube.com/video/LJjUME0eG6g/edit</t>
+        </is>
+      </c>
+      <c r="G184" s="7" t="inlineStr">
+        <is>
+          <t>📜 Теодос из Рима в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/485?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H184" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/BVYplCpF02c</t>
+          <t>https://youtu.be/LJjUME0eG6g</t>
         </is>
       </c>
       <c r="I184" s="2" t="n">
-        <v>686</v>
+        <v>458</v>
       </c>
       <c r="J184" s="2" t="n"/>
     </row>
@@ -8242,40 +8242,40 @@
         <v>184</v>
       </c>
       <c r="B185" s="3" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>עברית</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t>רבי אלעזר מגרמייזא (בעל הרוקח)</t>
-        </is>
-      </c>
-      <c r="E185" s="7" t="inlineStr">
-        <is>
-          <t>Rabbi Eleazar of Worms and the Ordinances of ShUM</t>
+          <t>הרב יצחק יעקב ריינס</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>הרב יצחק יעקב ריינס ומייסד המזרחי</t>
         </is>
       </c>
       <c r="F185" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/XewrhViUp7E/edit</t>
-        </is>
-      </c>
-      <c r="G185" s="7" t="inlineStr">
-        <is>
-          <t>📜 Rabbi Elazar of Worms (the Rokeach) on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/280?utm_source=youtube&amp;utm_medium=video</t>
+          <t>https://studio.youtube.com/video/BVYplCpF02c/edit</t>
+        </is>
+      </c>
+      <c r="G185" s="5" t="inlineStr">
+        <is>
+          <t>📜 הרב יצחק יעקב ריינס באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/489?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H185" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/XewrhViUp7E</t>
+          <t>https://youtu.be/BVYplCpF02c</t>
         </is>
       </c>
       <c r="I185" s="2" t="n">
-        <v>264</v>
+        <v>686</v>
       </c>
       <c r="J185" s="2" t="n"/>
     </row>
@@ -8293,31 +8293,31 @@
       </c>
       <c r="D186" s="4" t="inlineStr">
         <is>
-          <t>רבנו בחיי אבן פקודה – חובות הלבבות</t>
+          <t>ילקוט שמעוני</t>
         </is>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>“Duties of the Heart”: The Essence of Jewish Ethics</t>
+          <t>Yalkut Shimoni – the book that introduced nothing new, yet saved an entire world</t>
         </is>
       </c>
       <c r="F186" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/k5g7dfUeBlw/edit</t>
+          <t>https://studio.youtube.com/video/nAV7hB3__Lk/edit</t>
         </is>
       </c>
       <c r="G186" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbenu Bachya ibn Paquda (Duties of the Heart) on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/39?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Yalkut Shimoni on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/55?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H186" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/k5g7dfUeBlw</t>
+          <t>https://youtu.be/nAV7hB3__Lk</t>
         </is>
       </c>
       <c r="I186" s="2" t="n">
-        <v>480</v>
+        <v>402</v>
       </c>
       <c r="J186" s="2" t="n"/>
     </row>
@@ -8326,7 +8326,7 @@
         <v>186</v>
       </c>
       <c r="B187" s="3" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
@@ -8335,31 +8335,31 @@
       </c>
       <c r="D187" s="4" t="inlineStr">
         <is>
-          <t>ילקוט שמעוני</t>
+          <t>רבנו בחיי אבן פקודה – חובות הלבבות</t>
         </is>
       </c>
       <c r="E187" s="7" t="inlineStr">
         <is>
-          <t>Yalkut Shimoni – the book that introduced nothing new, yet saved an entire world</t>
+          <t>“Duties of the Heart”: The Essence of Jewish Ethics</t>
         </is>
       </c>
       <c r="F187" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/nAV7hB3__Lk/edit</t>
+          <t>https://studio.youtube.com/video/k5g7dfUeBlw/edit</t>
         </is>
       </c>
       <c r="G187" s="7" t="inlineStr">
         <is>
-          <t>📜 Yalkut Shimoni on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/55?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbenu Bachya ibn Paquda (Duties of the Heart) on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/39?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H187" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/nAV7hB3__Lk</t>
+          <t>https://youtu.be/k5g7dfUeBlw</t>
         </is>
       </c>
       <c r="I187" s="2" t="n">
-        <v>402</v>
+        <v>480</v>
       </c>
       <c r="J187" s="2" t="n"/>
     </row>
@@ -8498,36 +8498,36 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D191" s="4" t="inlineStr">
         <is>
-          <t>רפרם בר פפא</t>
+          <t>רבי אברהם בן שלמה הלוי בוקראט</t>
         </is>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
-          <t>Rafram bar Pappa - The Amora Who Connected Halakha, Science, and the Destruction of the Temple</t>
+          <t>Рабби Авраам Бократ - мудрец, изгнанный из Испании и выступивший в защиту РашиРабби Ав</t>
         </is>
       </c>
       <c r="F191" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/F970V-O0D_M/edit</t>
+          <t>https://studio.youtube.com/video/llK6TjhR-ok/edit</t>
         </is>
       </c>
       <c r="G191" s="7" t="inlineStr">
         <is>
-          <t>📜 Rafram bar Pappa on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/552?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Авраам бен Шломо а-Леви Букрат в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/627?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H191" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/F970V-O0D_M</t>
+          <t>https://youtu.be/llK6TjhR-ok</t>
         </is>
       </c>
       <c r="I191" s="2" t="n">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="J191" s="2" t="n"/>
     </row>
@@ -8540,36 +8540,36 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D192" s="4" t="inlineStr">
         <is>
-          <t>הצמח צדק (רבי מנחם מנדל שניאורסון)</t>
+          <t>רפרם בר פפא</t>
         </is>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>Цемах Цедек - Ребе, превративший Хабад в центр Галахи и духовного руководства</t>
+          <t>Rafram bar Pappa - The Amora Who Connected Halakha, Science, and the Destruction of the Temple</t>
         </is>
       </c>
       <c r="F192" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/27qzVovmga0/edit</t>
+          <t>https://studio.youtube.com/video/F970V-O0D_M/edit</t>
         </is>
       </c>
       <c r="G192" s="7" t="inlineStr">
         <is>
-          <t>📜 Цемах Цедек в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/501?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rafram bar Pappa on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/552?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H192" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/27qzVovmga0</t>
+          <t>https://youtu.be/F970V-O0D_M</t>
         </is>
       </c>
       <c r="I192" s="2" t="n">
-        <v>142</v>
+        <v>44</v>
       </c>
       <c r="J192" s="2" t="n"/>
     </row>
@@ -8582,36 +8582,36 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D193" s="4" t="inlineStr">
         <is>
-          <t>רבנו תם (ר׳ יעקב בן מאיר) – מהפכן השיטה התוספתית</t>
+          <t>הצמח צדק (רבי מנחם מנדל שניאורסון)</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr">
         <is>
-          <t>Rabbeinu Tam: Architect of Talmudic Scholarship and the Tosafists’ Legacy</t>
+          <t>Цемах Цедек - Ребе, превративший Хабад в центр Галахи и духовного руководства</t>
         </is>
       </c>
       <c r="F193" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/s0OXFxwzbvY/edit</t>
+          <t>https://studio.youtube.com/video/27qzVovmga0/edit</t>
         </is>
       </c>
       <c r="G193" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbenu Tam (R. Yaakov ben Meir) on Ozar Chachamim — the full research and his teachers and students: https://ozar-chachamim-app.vercel.app/en/sage/33?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Цемах Цедек в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/501?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H193" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/s0OXFxwzbvY</t>
+          <t>https://youtu.be/27qzVovmga0</t>
         </is>
       </c>
       <c r="I193" s="2" t="n">
-        <v>462</v>
+        <v>142</v>
       </c>
       <c r="J193" s="2" t="n"/>
     </row>
@@ -8620,40 +8620,40 @@
         <v>193</v>
       </c>
       <c r="B194" s="3" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D194" s="4" t="inlineStr">
         <is>
-          <t>רבי אברהם בן שלמה הלוי בוקראט</t>
+          <t>רבנו תם (ר׳ יעקב בן מאיר) – מהפכן השיטה התוספתית</t>
         </is>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>Рабби Авраам Бократ - мудрец, изгнанный из Испании и выступивший в защиту РашиРабби Ав</t>
+          <t>Rabbeinu Tam: Architect of Talmudic Scholarship and the Tosafists’ Legacy</t>
         </is>
       </c>
       <c r="F194" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/llK6TjhR-ok/edit</t>
+          <t>https://studio.youtube.com/video/s0OXFxwzbvY/edit</t>
         </is>
       </c>
       <c r="G194" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Авраам бен Шломо а-Леви Букрат в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/627?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbenu Tam (R. Yaakov ben Meir) on Ozar Chachamim — the full research and his teachers and students: https://ozar-chachamim-app.vercel.app/en/sage/33?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H194" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/llK6TjhR-ok</t>
+          <t>https://youtu.be/s0OXFxwzbvY</t>
         </is>
       </c>
       <c r="I194" s="2" t="n">
-        <v>7</v>
+        <v>462</v>
       </c>
       <c r="J194" s="2" t="n"/>
     </row>
@@ -8662,40 +8662,40 @@
         <v>194</v>
       </c>
       <c r="B195" s="3" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D195" s="4" t="inlineStr">
         <is>
-          <t>רבי יעקב פולק</t>
+          <t>הרב מרדכי שרעבי</t>
         </is>
       </c>
       <c r="E195" s="7" t="inlineStr">
         <is>
-          <t>Рабби Яаков Поллак: основатель метода пилпула и зарождения мира Торы в Польше</t>
+          <t>Biography of Rabbi Mordechai Sharabi, Kabbalist</t>
         </is>
       </c>
       <c r="F195" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/L5T6oVKBsSU/edit</t>
+          <t>https://studio.youtube.com/video/UP9MKbxXoUw/edit</t>
         </is>
       </c>
       <c r="G195" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Яаков Поллак в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/457?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Mordechai Sharabi on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/154?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H195" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/L5T6oVKBsSU</t>
+          <t>https://youtu.be/UP9MKbxXoUw</t>
         </is>
       </c>
       <c r="I195" s="2" t="n">
-        <v>169</v>
+        <v>616</v>
       </c>
       <c r="J195" s="2" t="n"/>
     </row>
@@ -8713,31 +8713,31 @@
       </c>
       <c r="D196" s="4" t="inlineStr">
         <is>
-          <t>הר"ן (רבנו נסים מגירונה)</t>
+          <t>רבי יעקב פולק</t>
         </is>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>Рабби Ниссим из Гироны (Ран): лидерство, галаха и философия в испанском иудаизме</t>
+          <t>Рабби Яаков Поллак: основатель метода пилпула и зарождения мира Торы в Польше</t>
         </is>
       </c>
       <c r="F196" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/h0NH3WSv5YA/edit</t>
+          <t>https://studio.youtube.com/video/L5T6oVKBsSU/edit</t>
         </is>
       </c>
       <c r="G196" s="7" t="inlineStr">
         <is>
-          <t>📜 Ран (рабейну Ниссим из Жироны) в «Оцар Хахамим» — полное исследование и его ученики: https://ozar-chachamim-app.vercel.app/ru/sage/13?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Яаков Поллак в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/457?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H196" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/h0NH3WSv5YA</t>
+          <t>https://youtu.be/L5T6oVKBsSU</t>
         </is>
       </c>
       <c r="I196" s="2" t="n">
-        <v>352</v>
+        <v>169</v>
       </c>
       <c r="J196" s="2" t="n"/>
     </row>
@@ -8750,36 +8750,36 @@
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D197" s="4" t="inlineStr">
         <is>
-          <t>הרב שלום שרעבי (הרש"ש)</t>
+          <t>הר"ן (רבנו נסים מגירונה)</t>
         </is>
       </c>
       <c r="E197" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Shalom Sharabi: The Father of Sephardic Kabbalists and the World of Kavanot</t>
+          <t>Рабби Ниссим из Гироны (Ран): лидерство, галаха и философия в испанском иудаизме</t>
         </is>
       </c>
       <c r="F197" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/HvMt-duFwZA/edit</t>
+          <t>https://studio.youtube.com/video/h0NH3WSv5YA/edit</t>
         </is>
       </c>
       <c r="G197" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Shalom Sharabi (the Rashash) on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/96?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Ран (рабейну Ниссим из Жироны) в «Оцар Хахамим» — полное исследование и его ученики: https://ozar-chachamim-app.vercel.app/ru/sage/13?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H197" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/HvMt-duFwZA</t>
+          <t>https://youtu.be/h0NH3WSv5YA</t>
         </is>
       </c>
       <c r="I197" s="2" t="n">
-        <v>553</v>
+        <v>352</v>
       </c>
       <c r="J197" s="2" t="n"/>
     </row>
@@ -8797,31 +8797,31 @@
       </c>
       <c r="D198" s="4" t="inlineStr">
         <is>
-          <t>הרב מרדכי שרעבי</t>
+          <t>הרב שלום שרעבי (הרש"ש)</t>
         </is>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>Biography of Rabbi Mordechai Sharabi, Kabbalist</t>
+          <t>Rabbi Shalom Sharabi: The Father of Sephardic Kabbalists and the World of Kavanot</t>
         </is>
       </c>
       <c r="F198" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/UP9MKbxXoUw/edit</t>
+          <t>https://studio.youtube.com/video/HvMt-duFwZA/edit</t>
         </is>
       </c>
       <c r="G198" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Mordechai Sharabi on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/154?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Shalom Sharabi (the Rashash) on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/96?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H198" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/UP9MKbxXoUw</t>
+          <t>https://youtu.be/HvMt-duFwZA</t>
         </is>
       </c>
       <c r="I198" s="2" t="n">
-        <v>616</v>
+        <v>553</v>
       </c>
       <c r="J198" s="2" t="n"/>
     </row>
@@ -10300,7 +10300,7 @@
         <v>233</v>
       </c>
       <c r="B234" s="3" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
@@ -10309,31 +10309,31 @@
       </c>
       <c r="D234" s="4" t="inlineStr">
         <is>
-          <t>הרב ד״ר אברהם לבני</t>
+          <t>הרב שמואל בורנשטיין – בעל 'שם משמואל'</t>
         </is>
       </c>
       <c r="E234" s="7" t="inlineStr">
         <is>
-          <t>Abraham Livni: The Israeli Secret and the Message to the World</t>
+          <t>Rabbi Shmuel Bornsztain - The Rebbe Whose Embrace Defied Death</t>
         </is>
       </c>
       <c r="F234" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/7xG6akhghaE/edit</t>
+          <t>https://studio.youtube.com/video/p4s-C-bZxak/edit</t>
         </is>
       </c>
       <c r="G234" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Dr. Avraham Livni on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/456?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Shmuel Bornsztain (the Shem MiShmuel) on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/131?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H234" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/7xG6akhghaE</t>
+          <t>https://youtu.be/p4s-C-bZxak</t>
         </is>
       </c>
       <c r="I234" s="2" t="n">
-        <v>172</v>
+        <v>665</v>
       </c>
       <c r="J234" s="2" t="n"/>
     </row>
@@ -10346,36 +10346,36 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D235" s="4" t="inlineStr">
         <is>
-          <t>גירוש ספרד</t>
+          <t>הרב ד״ר אברהם לבני</t>
         </is>
       </c>
       <c r="E235" s="7" t="inlineStr">
         <is>
-          <t>Наследие сефардского еврейства: от изгнания к рассеянию и до наших дней</t>
+          <t>Abraham Livni: The Israeli Secret and the Message to the World</t>
         </is>
       </c>
       <c r="F235" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/AKaU3ACKg08/edit</t>
+          <t>https://studio.youtube.com/video/7xG6akhghaE/edit</t>
         </is>
       </c>
       <c r="G235" s="7" t="inlineStr">
         <is>
-          <t>📜 Изгнание из Испании в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/331?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Dr. Avraham Livni on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/456?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H235" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/AKaU3ACKg08</t>
+          <t>https://youtu.be/7xG6akhghaE</t>
         </is>
       </c>
       <c r="I235" s="2" t="n">
-        <v>308</v>
+        <v>172</v>
       </c>
       <c r="J235" s="2" t="n"/>
     </row>
@@ -10393,31 +10393,31 @@
       </c>
       <c r="D236" s="4" t="inlineStr">
         <is>
-          <t>יעקב בן אשר</t>
+          <t>גירוש ספרד</t>
         </is>
       </c>
       <c r="E236" s="7" t="inlineStr">
         <is>
-          <t>«Арбаа Турим» и Бааль ха-Турим: архитектура галахи и толкование Торы</t>
+          <t>Наследие сефардского еврейства: от изгнания к рассеянию и до наших дней</t>
         </is>
       </c>
       <c r="F236" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/kkcdpEijKKU/edit</t>
+          <t>https://studio.youtube.com/video/AKaU3ACKg08/edit</t>
         </is>
       </c>
       <c r="G236" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Яаков бен Ашер (Тур) в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/189?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Изгнание из Испании в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/331?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H236" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/kkcdpEijKKU</t>
+          <t>https://youtu.be/AKaU3ACKg08</t>
         </is>
       </c>
       <c r="I236" s="2" t="n">
-        <v>447</v>
+        <v>308</v>
       </c>
       <c r="J236" s="2" t="n"/>
     </row>
@@ -10430,36 +10430,36 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D237" s="4" t="inlineStr">
         <is>
-          <t>הרב שמואל בורנשטיין – בעל 'שם משמואל'</t>
+          <t>יעקב בן אשר</t>
         </is>
       </c>
       <c r="E237" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Shmuel Bornsztain - The Rebbe Whose Embrace Defied Death</t>
+          <t>«Арбаа Турим» и Бааль ха-Турим: архитектура галахи и толкование Торы</t>
         </is>
       </c>
       <c r="F237" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/p4s-C-bZxak/edit</t>
+          <t>https://studio.youtube.com/video/kkcdpEijKKU/edit</t>
         </is>
       </c>
       <c r="G237" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Shmuel Bornsztain (the Shem MiShmuel) on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/131?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Яаков бен Ашер (Тур) в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/189?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H237" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/p4s-C-bZxak</t>
+          <t>https://youtu.be/kkcdpEijKKU</t>
         </is>
       </c>
       <c r="I237" s="2" t="n">
-        <v>665</v>
+        <v>447</v>
       </c>
       <c r="J237" s="2" t="n"/>
     </row>
@@ -10603,31 +10603,31 @@
       </c>
       <c r="D241" s="4" t="inlineStr">
         <is>
-          <t>רבי אפרים אנקווה – 'הרב הרוכב על האריה'</t>
+          <t>הרב יהודה אלקלעי – תשובה שהופכת לתוכנית לאומית</t>
         </is>
       </c>
       <c r="E241" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Ephraim Ankawa: His Life and Legacy</t>
+          <t>Alkalai: The Harbinger of Political Zionism</t>
         </is>
       </c>
       <c r="F241" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/v9NtNryySZ0/edit</t>
+          <t>https://studio.youtube.com/video/dQ69FzKEc94/edit</t>
         </is>
       </c>
       <c r="G241" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Ephraim Ankawa on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/58?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Yehuda Alkalai on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/108?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H241" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/v9NtNryySZ0</t>
+          <t>https://youtu.be/dQ69FzKEc94</t>
         </is>
       </c>
       <c r="I241" s="2" t="n">
-        <v>671</v>
+        <v>486</v>
       </c>
       <c r="J241" s="2" t="n"/>
     </row>
@@ -10636,40 +10636,40 @@
         <v>241</v>
       </c>
       <c r="B242" s="3" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D242" s="4" t="inlineStr">
         <is>
-          <t>רבי יוסף ג'יקטיליה</t>
+          <t>רבי אפרים אנקווה – 'הרב הרוכב על האריה'</t>
         </is>
       </c>
       <c r="E242" s="7" t="inlineStr">
         <is>
-          <t>Рабби Йосеф Джикатилья: «Врата света» и тайны Божественного Имени</t>
+          <t>Rabbi Ephraim Ankawa: His Life and Legacy</t>
         </is>
       </c>
       <c r="F242" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/FCgf1OySW6Y/edit</t>
+          <t>https://studio.youtube.com/video/v9NtNryySZ0/edit</t>
         </is>
       </c>
       <c r="G242" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Йосеф Гикатилла в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/471?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Ephraim Ankawa on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/58?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H242" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/FCgf1OySW6Y</t>
+          <t>https://youtu.be/v9NtNryySZ0</t>
         </is>
       </c>
       <c r="I242" s="2" t="n">
-        <v>151</v>
+        <v>671</v>
       </c>
       <c r="J242" s="2" t="n"/>
     </row>
@@ -10682,36 +10682,36 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D243" s="4" t="inlineStr">
         <is>
-          <t>רבי מאיר בן ברוך הלוי (מהר״ם סג״ל)</t>
+          <t>רבי יוסף ג'יקטיליה</t>
         </is>
       </c>
       <c r="E243" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Meir ben Baruch HaLevi Segal – The Man Who Reshaped Ashkenazi Rabbinic Authority</t>
+          <t>Рабби Йосеф Джикатилья: «Врата света» и тайны Божественного Имени</t>
         </is>
       </c>
       <c r="F243" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/FBL394gsb4g/edit</t>
+          <t>https://studio.youtube.com/video/FCgf1OySW6Y/edit</t>
         </is>
       </c>
       <c r="G243" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Meir ben Baruch HaLevi (Maharam Segal) on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/425?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Йосеф Гикатилла в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/471?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H243" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/FBL394gsb4g</t>
+          <t>https://youtu.be/FCgf1OySW6Y</t>
         </is>
       </c>
       <c r="I243" s="2" t="n">
-        <v>202</v>
+        <v>151</v>
       </c>
       <c r="J243" s="2" t="n"/>
     </row>
@@ -10724,36 +10724,36 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D244" s="4" t="inlineStr">
         <is>
-          <t>חולדה הנביאה</t>
+          <t>רבי מאיר בן ברוך הלוי (מהר״ם סג״ל)</t>
         </is>
       </c>
       <c r="E244" s="7" t="inlineStr">
         <is>
-          <t>Пророчица Хульда — история открытия книги Торы в Храме</t>
+          <t>Rabbi Meir ben Baruch HaLevi Segal – The Man Who Reshaped Ashkenazi Rabbinic Authority</t>
         </is>
       </c>
       <c r="F244" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/FQ0SYVbT4y4/edit</t>
+          <t>https://studio.youtube.com/video/FBL394gsb4g/edit</t>
         </is>
       </c>
       <c r="G244" s="7" t="inlineStr">
         <is>
-          <t>📜 Пророчица Хульда в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/270?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Meir ben Baruch HaLevi (Maharam Segal) on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/425?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H244" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/FQ0SYVbT4y4</t>
+          <t>https://youtu.be/FBL394gsb4g</t>
         </is>
       </c>
       <c r="I244" s="2" t="n">
-        <v>273</v>
+        <v>202</v>
       </c>
       <c r="J244" s="2" t="n"/>
     </row>
@@ -10766,36 +10766,36 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D245" s="4" t="inlineStr">
         <is>
-          <t>רבי שלמה הלוי אלקבץ</t>
+          <t>חולדה הנביאה</t>
         </is>
       </c>
       <c r="E245" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Shlomo Alkabetz: Architect of Kabbalah, Shabbat, and Liturgical Poetry in Safed</t>
+          <t>Пророчица Хульда — история открытия книги Торы в Храме</t>
         </is>
       </c>
       <c r="F245" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/0Grw9xmokQs/edit</t>
+          <t>https://studio.youtube.com/video/FQ0SYVbT4y4/edit</t>
         </is>
       </c>
       <c r="G245" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Shlomo HaLevi Alkabetz on Ozar Chachamim — the full research and his teachers and students: https://ozar-chachamim-app.vercel.app/en/sage/327?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Пророчица Хульда в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/270?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H245" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/0Grw9xmokQs</t>
+          <t>https://youtu.be/FQ0SYVbT4y4</t>
         </is>
       </c>
       <c r="I245" s="2" t="n">
-        <v>336</v>
+        <v>273</v>
       </c>
       <c r="J245" s="2" t="n"/>
     </row>
@@ -10808,36 +10808,36 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D246" s="4" t="inlineStr">
         <is>
-          <t>הרב אברהם יהושע השל – הגות ומעורבות מוסרית</t>
+          <t>רבי שלמה הלוי אלקבץ</t>
         </is>
       </c>
       <c r="E246" s="7" t="inlineStr">
         <is>
-          <t>Раввин Авраам Джошуа Хешель — философия, нравственная ответственность и человеческая вовлечённость</t>
+          <t>Rabbi Shlomo Alkabetz: Architect of Kabbalah, Shabbat, and Liturgical Poetry in Safed</t>
         </is>
       </c>
       <c r="F246" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/ASOGLLfZ_DE/edit</t>
+          <t>https://studio.youtube.com/video/0Grw9xmokQs/edit</t>
         </is>
       </c>
       <c r="G246" s="7" t="inlineStr">
         <is>
-          <t>📜 Рав Авраам Йехошуа Хешель в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/152?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Shlomo HaLevi Alkabetz on Ozar Chachamim — the full research and his teachers and students: https://ozar-chachamim-app.vercel.app/en/sage/327?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H246" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/ASOGLLfZ_DE</t>
+          <t>https://youtu.be/0Grw9xmokQs</t>
         </is>
       </c>
       <c r="I246" s="2" t="n">
-        <v>468</v>
+        <v>336</v>
       </c>
       <c r="J246" s="2" t="n"/>
     </row>
@@ -10850,36 +10850,36 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D247" s="4" t="inlineStr">
         <is>
-          <t>הרב יהודה אלקלעי – תשובה שהופכת לתוכנית לאומית</t>
+          <t>הרב אברהם יהושע השל – הגות ומעורבות מוסרית</t>
         </is>
       </c>
       <c r="E247" s="7" t="inlineStr">
         <is>
-          <t>Alkalai: The Harbinger of Political Zionism</t>
+          <t>Раввин Авраам Джошуа Хешель — философия, нравственная ответственность и человеческая вовлечённость</t>
         </is>
       </c>
       <c r="F247" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/dQ69FzKEc94/edit</t>
+          <t>https://studio.youtube.com/video/ASOGLLfZ_DE/edit</t>
         </is>
       </c>
       <c r="G247" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Yehuda Alkalai on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/108?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рав Авраам Йехошуа Хешель в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/152?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H247" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/dQ69FzKEc94</t>
+          <t>https://youtu.be/ASOGLLfZ_DE</t>
         </is>
       </c>
       <c r="I247" s="2" t="n">
-        <v>486</v>
+        <v>468</v>
       </c>
       <c r="J247" s="2" t="n"/>
     </row>
@@ -14336,36 +14336,36 @@
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>רבי חיים מוולוז'ין – מייסד 'אם הישיבות' ו'נפש החיים'</t>
+          <t>רבי יוסף אלבו</t>
         </is>
       </c>
       <c r="E330" s="7" t="inlineStr">
         <is>
-          <t>Рабби Хаим из Воложина — тихий революционер, сформировавший позвоночник мира Торы</t>
+          <t>Rabbi Joseph Albo – The Sage Who Preserved Faith in a Time of Crisis</t>
         </is>
       </c>
       <c r="F330" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/D5ctLfiF46Q/edit</t>
+          <t>https://studio.youtube.com/video/gmQs0iEFQo0/edit</t>
         </is>
       </c>
       <c r="G330" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Хаим из Воложина в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/99?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Yosef Albo on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/17?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H330" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/D5ctLfiF46Q</t>
+          <t>https://youtu.be/gmQs0iEFQo0</t>
         </is>
       </c>
       <c r="I330" s="2" t="n">
-        <v>657</v>
+        <v>594</v>
       </c>
       <c r="J330" s="2" t="n"/>
     </row>
@@ -14374,40 +14374,40 @@
         <v>330</v>
       </c>
       <c r="B331" s="3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr">
         <is>
-          <t>צרויה</t>
+          <t>רבי חיים מוולוז'ין – מייסד 'אם הישיבות' ו'נפש החיים'</t>
         </is>
       </c>
       <c r="E331" s="7" t="inlineStr">
         <is>
-          <t>Zeruiah - The Woman Whose Sons Bore Her Name at the Heart of David’s Kingdom</t>
+          <t>Рабби Хаим из Воложина — тихий революционер, сформировавший позвоночник мира Торы</t>
         </is>
       </c>
       <c r="F331" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/VbKKhrAATyE/edit</t>
+          <t>https://studio.youtube.com/video/D5ctLfiF46Q/edit</t>
         </is>
       </c>
       <c r="G331" s="7" t="inlineStr">
         <is>
-          <t>📜 Zeruiah on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/535?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Хаим из Воложина в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/99?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H331" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/VbKKhrAATyE</t>
+          <t>https://youtu.be/D5ctLfiF46Q</t>
         </is>
       </c>
       <c r="I331" s="2" t="n">
-        <v>50</v>
+        <v>657</v>
       </c>
       <c r="J331" s="2" t="n"/>
     </row>
@@ -14425,31 +14425,31 @@
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>דונה גרציה נשיא</t>
+          <t>צרויה</t>
         </is>
       </c>
       <c r="E332" s="7" t="inlineStr">
         <is>
-          <t>Dona Gracia Nasi - The Woman Who Turned Wealth and Political Power into a Jewish Rescue Mission</t>
+          <t>Zeruiah - The Woman Whose Sons Bore Her Name at the Heart of David’s Kingdom</t>
         </is>
       </c>
       <c r="F332" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/xQ2dUpSvXYU/edit</t>
+          <t>https://studio.youtube.com/video/VbKKhrAATyE/edit</t>
         </is>
       </c>
       <c r="G332" s="7" t="inlineStr">
         <is>
-          <t>📜 Doña Gracia Nasi on Ozar Chachamim — the full research and a quiz: https://ozar-chachamim-app.vercel.app/en/sage/524?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Zeruiah on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/535?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H332" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/xQ2dUpSvXYU</t>
+          <t>https://youtu.be/VbKKhrAATyE</t>
         </is>
       </c>
       <c r="I332" s="2" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="J332" s="2" t="n"/>
     </row>
@@ -14467,31 +14467,31 @@
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>רבי גדליה נדל</t>
+          <t>דונה גרציה נשיא</t>
         </is>
       </c>
       <c r="E333" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Gedaliah Nadel - Torah, Science, and the Search for Truth</t>
+          <t>Dona Gracia Nasi - The Woman Who Turned Wealth and Political Power into a Jewish Rescue Mission</t>
         </is>
       </c>
       <c r="F333" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/b3MGed9-cb0/edit</t>
+          <t>https://studio.youtube.com/video/xQ2dUpSvXYU/edit</t>
         </is>
       </c>
       <c r="G333" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Gedalia Nadel on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/541?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Doña Gracia Nasi on Ozar Chachamim — the full research and a quiz: https://ozar-chachamim-app.vercel.app/en/sage/524?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H333" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/b3MGed9-cb0</t>
+          <t>https://youtu.be/xQ2dUpSvXYU</t>
         </is>
       </c>
       <c r="I333" s="2" t="n">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="J333" s="2" t="n"/>
     </row>
@@ -14504,7 +14504,7 @@
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
@@ -14514,26 +14514,26 @@
       </c>
       <c r="E334" s="7" t="inlineStr">
         <is>
-          <t>Раввин Гедалия Надель - Тора, наука и поиск истины</t>
+          <t>Rabbi Gedaliah Nadel - Torah, Science, and the Search for Truth</t>
         </is>
       </c>
       <c r="F334" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/VC4hexRfopM/edit</t>
+          <t>https://studio.youtube.com/video/b3MGed9-cb0/edit</t>
         </is>
       </c>
       <c r="G334" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Гедалья Надель в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/541?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Gedalia Nadel on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/541?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H334" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/VC4hexRfopM</t>
+          <t>https://youtu.be/b3MGed9-cb0</t>
         </is>
       </c>
       <c r="I334" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J334" s="2" t="n"/>
     </row>
@@ -14551,31 +14551,31 @@
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>רבי יחיאל בן יקותיאל ענו</t>
+          <t>רבי גדליה נדל</t>
         </is>
       </c>
       <c r="E335" s="7" t="inlineStr">
         <is>
-          <t>Рабби Йехиэль бен Йекутиэль: Лейденская рукопись</t>
+          <t>Раввин Гедалия Надель - Тора, наука и поиск истины</t>
         </is>
       </c>
       <c r="F335" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/BX0hmaRuQm0/edit</t>
+          <t>https://studio.youtube.com/video/VC4hexRfopM/edit</t>
         </is>
       </c>
       <c r="G335" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Йехиэль бен Йекутиэль Анав в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/397?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Гедалья Надель в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/541?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H335" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/BX0hmaRuQm0</t>
+          <t>https://youtu.be/VC4hexRfopM</t>
         </is>
       </c>
       <c r="I335" s="2" t="n">
-        <v>241</v>
+        <v>76</v>
       </c>
       <c r="J335" s="2" t="n"/>
     </row>
@@ -14593,31 +14593,31 @@
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>הרב עובדיה הדאיה</t>
+          <t>רבי יחיאל בן יקותיאל ענו</t>
         </is>
       </c>
       <c r="E336" s="7" t="inlineStr">
         <is>
-          <t>Рав Овадия Адая: опора галахического учения, каббалы и сионизма</t>
+          <t>Рабби Йехиэль бен Йекутиэль: Лейденская рукопись</t>
         </is>
       </c>
       <c r="F336" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/TavL4Mjk7g0/edit</t>
+          <t>https://studio.youtube.com/video/BX0hmaRuQm0/edit</t>
         </is>
       </c>
       <c r="G336" s="7" t="inlineStr">
         <is>
-          <t>📜 Рав Овадья Хадая в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/144?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Йехиэль бен Йекутиэль Анав в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/397?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H336" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/TavL4Mjk7g0</t>
+          <t>https://youtu.be/BX0hmaRuQm0</t>
         </is>
       </c>
       <c r="I336" s="2" t="n">
-        <v>368</v>
+        <v>241</v>
       </c>
       <c r="J336" s="2" t="n"/>
     </row>
@@ -14630,36 +14630,36 @@
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>הרב יצחק אלפייה</t>
+          <t>הרב עובדיה הדאיה</t>
         </is>
       </c>
       <c r="E337" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Yitzhak Alfiya: His Teachings and Legacy</t>
+          <t>Рав Овадия Адая: опора галахического учения, каббалы и сионизма</t>
         </is>
       </c>
       <c r="F337" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/Z2ywjHTTFuE/edit</t>
+          <t>https://studio.youtube.com/video/TavL4Mjk7g0/edit</t>
         </is>
       </c>
       <c r="G337" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Yitzchak Alfiya on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/137?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рав Овадья Хадая в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/144?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H337" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/Z2ywjHTTFuE</t>
+          <t>https://youtu.be/TavL4Mjk7g0</t>
         </is>
       </c>
       <c r="I337" s="2" t="n">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="J337" s="2" t="n"/>
     </row>
@@ -14677,31 +14677,31 @@
       </c>
       <c r="D338" s="4" t="inlineStr">
         <is>
-          <t>הראבי"ה (רבי אליעזר בן יואל הלוי)</t>
+          <t>הרב יצחק אלפייה</t>
         </is>
       </c>
       <c r="E338" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Eliezer ben Joel HaLevi (Ra’avyah): His Legacy, Halakhic Authority, and Life Story</t>
+          <t>Rabbi Yitzhak Alfiya: His Teachings and Legacy</t>
         </is>
       </c>
       <c r="F338" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/RDA9SnI7ZD0/edit</t>
+          <t>https://studio.youtube.com/video/Z2ywjHTTFuE/edit</t>
         </is>
       </c>
       <c r="G338" s="7" t="inlineStr">
         <is>
-          <t>📜 The Ra'avia on Ozar Chachamim — the full research and his teachers and students: https://ozar-chachamim-app.vercel.app/en/sage/49?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Yitzchak Alfiya on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/137?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H338" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/RDA9SnI7ZD0</t>
+          <t>https://youtu.be/Z2ywjHTTFuE</t>
         </is>
       </c>
       <c r="I338" s="2" t="n">
-        <v>397</v>
+        <v>370</v>
       </c>
       <c r="J338" s="2" t="n"/>
     </row>
@@ -14714,36 +14714,36 @@
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D339" s="4" t="inlineStr">
         <is>
-          <t>הבן איש חי (רבי יוסף חיים מבגדד)</t>
+          <t>הראבי"ה (רבי אליעזר בן יואל הלוי)</t>
         </is>
       </c>
       <c r="E339" s="7" t="inlineStr">
         <is>
-          <t>Рабби Йосеф Хаим из Багдада: учение, социальная критика и наследие</t>
+          <t>Rabbi Eliezer ben Joel HaLevi (Ra’avyah): His Legacy, Halakhic Authority, and Life Story</t>
         </is>
       </c>
       <c r="F339" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/ST3uDsJdluA/edit</t>
+          <t>https://studio.youtube.com/video/RDA9SnI7ZD0/edit</t>
         </is>
       </c>
       <c r="G339" s="7" t="inlineStr">
         <is>
-          <t>📜 Бен Иш Хай в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/126?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 The Ra'avia on Ozar Chachamim — the full research and his teachers and students: https://ozar-chachamim-app.vercel.app/en/sage/49?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H339" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/ST3uDsJdluA</t>
+          <t>https://youtu.be/RDA9SnI7ZD0</t>
         </is>
       </c>
       <c r="I339" s="2" t="n">
-        <v>485</v>
+        <v>397</v>
       </c>
       <c r="J339" s="2" t="n"/>
     </row>
@@ -14756,36 +14756,36 @@
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D340" s="4" t="inlineStr">
         <is>
-          <t>רבי יוסף אלבו</t>
+          <t>הבן איש חי (רבי יוסף חיים מבגדד)</t>
         </is>
       </c>
       <c r="E340" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Joseph Albo – The Sage Who Preserved Faith in a Time of Crisis</t>
+          <t>Рабби Йосеф Хаим из Багдада: учение, социальная критика и наследие</t>
         </is>
       </c>
       <c r="F340" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/gmQs0iEFQo0/edit</t>
+          <t>https://studio.youtube.com/video/ST3uDsJdluA/edit</t>
         </is>
       </c>
       <c r="G340" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Yosef Albo on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/17?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Бен Иш Хай в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/126?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H340" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/gmQs0iEFQo0</t>
+          <t>https://youtu.be/ST3uDsJdluA</t>
         </is>
       </c>
       <c r="I340" s="2" t="n">
-        <v>594</v>
+        <v>485</v>
       </c>
       <c r="J340" s="2" t="n"/>
     </row>
@@ -18037,31 +18037,31 @@
       </c>
       <c r="D418" s="4" t="inlineStr">
         <is>
-          <t>הרמ״ע מפאנו</t>
+          <t>שרה אמנו</t>
         </is>
       </c>
       <c r="E418" s="7" t="inlineStr">
         <is>
-          <t>The Teachings and Historical Influence of Rabbi Menachem Azariah of Pano</t>
+          <t>Sarah Our Matriarch:The Foundation of Prophecy and the Sovereignty of Spirit in the Tent and in Time</t>
         </is>
       </c>
       <c r="F418" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/coQyIiMtHho/edit</t>
+          <t>https://studio.youtube.com/video/QHHa6EXkb8U/edit</t>
         </is>
       </c>
       <c r="G418" s="7" t="inlineStr">
         <is>
-          <t>📜 The Rama of Fano (Rabbi Menachem Azariah) on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/439?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Sarah Our Matriarch on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/448?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H418" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/coQyIiMtHho</t>
+          <t>https://youtu.be/QHHa6EXkb8U</t>
         </is>
       </c>
       <c r="I418" s="2" t="n">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="J418" s="2" t="n"/>
     </row>
@@ -18079,31 +18079,31 @@
       </c>
       <c r="D419" s="4" t="inlineStr">
         <is>
-          <t>חנה הנביאה</t>
+          <t>הרמ״ע מפאנו</t>
         </is>
       </c>
       <c r="E419" s="7" t="inlineStr">
         <is>
-          <t>Hannah’s Prayer: Faith, Halakha, and a Model for Education</t>
+          <t>The Teachings and Historical Influence of Rabbi Menachem Azariah of Pano</t>
         </is>
       </c>
       <c r="F419" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/uf6D-8ElhLQ/edit</t>
+          <t>https://studio.youtube.com/video/coQyIiMtHho/edit</t>
         </is>
       </c>
       <c r="G419" s="7" t="inlineStr">
         <is>
-          <t>📜 Hannah the Prophetess on Ozar Chachamim — the full research and a quiz: https://ozar-chachamim-app.vercel.app/en/sage/282?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 The Rama of Fano (Rabbi Menachem Azariah) on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/439?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H419" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/uf6D-8ElhLQ</t>
+          <t>https://youtu.be/coQyIiMtHho</t>
         </is>
       </c>
       <c r="I419" s="2" t="n">
-        <v>262</v>
+        <v>185</v>
       </c>
       <c r="J419" s="2" t="n"/>
     </row>
@@ -18121,31 +18121,31 @@
       </c>
       <c r="D420" s="4" t="inlineStr">
         <is>
-          <t>רבי יהונתן הכהן מלוניל</t>
+          <t>חנה הנביאה</t>
         </is>
       </c>
       <c r="E420" s="7" t="inlineStr">
         <is>
-          <t>The Great Luminary of Lunel: The Sage Who Brought Maimonides to Europe</t>
+          <t>Hannah’s Prayer: Faith, Halakha, and a Model for Education</t>
         </is>
       </c>
       <c r="F420" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/YxI2_lApcDI/edit</t>
+          <t>https://studio.youtube.com/video/uf6D-8ElhLQ/edit</t>
         </is>
       </c>
       <c r="G420" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Yehonatan HaKohen of Lunel on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/278?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Hannah the Prophetess on Ozar Chachamim — the full research and a quiz: https://ozar-chachamim-app.vercel.app/en/sage/282?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H420" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/YxI2_lApcDI</t>
+          <t>https://youtu.be/uf6D-8ElhLQ</t>
         </is>
       </c>
       <c r="I420" s="2" t="n">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="J420" s="2" t="n"/>
     </row>
@@ -18163,31 +18163,31 @@
       </c>
       <c r="D421" s="4" t="inlineStr">
         <is>
-          <t>הרב שלמה זלמן אויערבך</t>
+          <t>רבי יהונתן הכהן מלוניל</t>
         </is>
       </c>
       <c r="E421" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Shlomo Zalman Auerbach: A Leading Halachic Authority in the Modern Era</t>
+          <t>The Great Luminary of Lunel: The Sage Who Brought Maimonides to Europe</t>
         </is>
       </c>
       <c r="F421" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/WvYmgdvQa2M/edit</t>
+          <t>https://studio.youtube.com/video/YxI2_lApcDI/edit</t>
         </is>
       </c>
       <c r="G421" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Shlomo Zalman Auerbach on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/157?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Yehonatan HaKohen of Lunel on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/278?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H421" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/WvYmgdvQa2M</t>
+          <t>https://youtu.be/YxI2_lApcDI</t>
         </is>
       </c>
       <c r="I421" s="2" t="n">
-        <v>391</v>
+        <v>267</v>
       </c>
       <c r="J421" s="2" t="n"/>
     </row>
@@ -18205,31 +18205,31 @@
       </c>
       <c r="D422" s="4" t="inlineStr">
         <is>
-          <t>הרב אפרים נבון (1677–1735) – מחנה אפרים: עקרונות פסיקה וסדרי קניינים</t>
+          <t>הרב שלמה זלמן אויערבך</t>
         </is>
       </c>
       <c r="E422" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Ephraim Navon and Machaneh Ephraim</t>
+          <t>Rabbi Shlomo Zalman Auerbach: A Leading Halachic Authority in the Modern Era</t>
         </is>
       </c>
       <c r="F422" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/_8SN0I-7CoY/edit</t>
+          <t>https://studio.youtube.com/video/WvYmgdvQa2M/edit</t>
         </is>
       </c>
       <c r="G422" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Ephraim Navon on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/87?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Shlomo Zalman Auerbach on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/157?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H422" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/_8SN0I-7CoY</t>
+          <t>https://youtu.be/WvYmgdvQa2M</t>
         </is>
       </c>
       <c r="I422" s="2" t="n">
-        <v>521</v>
+        <v>391</v>
       </c>
       <c r="J422" s="2" t="n"/>
     </row>
@@ -18247,31 +18247,31 @@
       </c>
       <c r="D423" s="4" t="inlineStr">
         <is>
-          <t>הרב יצחק אבוהב</t>
+          <t>הרב אפרים נבון (1677–1735) – מחנה אפרים: עקרונות פסיקה וסדרי קניינים</t>
         </is>
       </c>
       <c r="E423" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Yitzhak Abuhav – The Light of Generations, Author of “Menorat Ha-Maor”</t>
+          <t>Rabbi Ephraim Navon and Machaneh Ephraim</t>
         </is>
       </c>
       <c r="F423" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/L03uSsP6N4E/edit</t>
+          <t>https://studio.youtube.com/video/_8SN0I-7CoY/edit</t>
         </is>
       </c>
       <c r="G423" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Yitzchak Aboab on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/62?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Ephraim Navon on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/87?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H423" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/L03uSsP6N4E</t>
+          <t>https://youtu.be/_8SN0I-7CoY</t>
         </is>
       </c>
       <c r="I423" s="2" t="n">
-        <v>604</v>
+        <v>521</v>
       </c>
       <c r="J423" s="2" t="n"/>
     </row>
@@ -18284,36 +18284,36 @@
       </c>
       <c r="C424" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D424" s="4" t="inlineStr">
         <is>
-          <t>רבי אפרים אנקווה – 'הרב הרוכב על האריה'</t>
+          <t>הרב יצחק אבוהב</t>
         </is>
       </c>
       <c r="E424" s="7" t="inlineStr">
         <is>
-          <t>Рав Эфраим Анкава: жизнь и деятельность</t>
+          <t>Rabbi Yitzhak Abuhav – The Light of Generations, Author of “Menorat Ha-Maor”</t>
         </is>
       </c>
       <c r="F424" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/4A2JxVeX8Yc/edit</t>
+          <t>https://studio.youtube.com/video/L03uSsP6N4E/edit</t>
         </is>
       </c>
       <c r="G424" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Эфраим Анкава в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/58?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Yitzchak Aboab on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/62?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H424" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/4A2JxVeX8Yc</t>
+          <t>https://youtu.be/L03uSsP6N4E</t>
         </is>
       </c>
       <c r="I424" s="2" t="n">
-        <v>672</v>
+        <v>604</v>
       </c>
       <c r="J424" s="2" t="n"/>
     </row>
@@ -18326,36 +18326,36 @@
       </c>
       <c r="C425" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D425" s="4" t="inlineStr">
         <is>
-          <t>שמואל (האמורא)</t>
+          <t>רבי אפרים אנקווה – 'הרב הרוכב על האריה'</t>
         </is>
       </c>
       <c r="E425" s="7" t="inlineStr">
         <is>
-          <t>Shmuel: His Legal Rulings and Teachings</t>
+          <t>Рав Эфраим Анкава: жизнь и деятельность</t>
         </is>
       </c>
       <c r="F425" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/6UfjwSUASjI/edit</t>
+          <t>https://studio.youtube.com/video/4A2JxVeX8Yc/edit</t>
         </is>
       </c>
       <c r="G425" s="7" t="inlineStr">
         <is>
-          <t>📜 Shmuel (the Amora) on Ozar Chachamim — the full research and his teachers and students: https://ozar-chachamim-app.vercel.app/en/sage/482?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Эфраим Анкава в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/58?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H425" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/6UfjwSUASjI</t>
+          <t>https://youtu.be/4A2JxVeX8Yc</t>
         </is>
       </c>
       <c r="I425" s="2" t="n">
-        <v>692</v>
+        <v>672</v>
       </c>
       <c r="J425" s="2" t="n"/>
     </row>
@@ -18364,40 +18364,40 @@
         <v>425</v>
       </c>
       <c r="B426" s="3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C426" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D426" s="4" t="inlineStr">
         <is>
-          <t>הרבנית חיה מושקא שניאורסון</t>
+          <t>שמואל (האמורא)</t>
         </is>
       </c>
       <c r="E426" s="7" t="inlineStr">
         <is>
-          <t>Ребецн Хая-Мушка Шнеерсон - духовное партнерство, самоотверженность и тихое лидерство</t>
+          <t>Shmuel: His Legal Rulings and Teachings</t>
         </is>
       </c>
       <c r="F426" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/vfjBSPWJqe4/edit</t>
+          <t>https://studio.youtube.com/video/6UfjwSUASjI/edit</t>
         </is>
       </c>
       <c r="G426" s="7" t="inlineStr">
         <is>
-          <t>📜 Ребецн Хая Мушка Шнеерсон в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/610?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Shmuel (the Amora) on Ozar Chachamim — the full research and his teachers and students: https://ozar-chachamim-app.vercel.app/en/sage/482?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H426" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/vfjBSPWJqe4</t>
+          <t>https://youtu.be/6UfjwSUASjI</t>
         </is>
       </c>
       <c r="I426" s="2" t="n">
-        <v>95</v>
+        <v>692</v>
       </c>
       <c r="J426" s="2" t="n"/>
     </row>
@@ -18410,36 +18410,36 @@
       </c>
       <c r="C427" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D427" s="4" t="inlineStr">
         <is>
-          <t>רבי שמשון בן אליעזר (ברוך שאמר)</t>
+          <t>הרבנית חיה מושקא שניאורסון</t>
         </is>
       </c>
       <c r="E427" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Samson ben Eliezer and the Tradition of Scribal Writing (STaM) in the Book "Baruch She’amar"</t>
+          <t>Ребецн Хая-Мушка Шнеерсон - духовное партнерство, самоотверженность и тихое лидерство</t>
         </is>
       </c>
       <c r="F427" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/nJQ_RbQIEvI/edit</t>
+          <t>https://studio.youtube.com/video/vfjBSPWJqe4/edit</t>
         </is>
       </c>
       <c r="G427" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Shimshon ben Eliezer (Baruch She'amar) on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/426?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Ребецн Хая Мушка Шнеерсон в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/610?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H427" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/nJQ_RbQIEvI</t>
+          <t>https://youtu.be/vfjBSPWJqe4</t>
         </is>
       </c>
       <c r="I427" s="2" t="n">
-        <v>200</v>
+        <v>95</v>
       </c>
       <c r="J427" s="2" t="n"/>
     </row>
@@ -18457,31 +18457,31 @@
       </c>
       <c r="D428" s="4" t="inlineStr">
         <is>
-          <t>רבי נחמן קרוכמל (רנ״ק)</t>
+          <t>רבי שמשון בן אליעזר (ברוך שאמר)</t>
         </is>
       </c>
       <c r="E428" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Nachman Krochmal (RaNaK) – The Thinker Who Turned History into Proof of the Eternity of Israel</t>
+          <t>Rabbi Samson ben Eliezer and the Tradition of Scribal Writing (STaM) in the Book "Baruch She’amar"</t>
         </is>
       </c>
       <c r="F428" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/oAjWELNrN0I/edit</t>
+          <t>https://studio.youtube.com/video/nJQ_RbQIEvI/edit</t>
         </is>
       </c>
       <c r="G428" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Nachman Krochmal (Ranak) on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/315?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Shimshon ben Eliezer (Baruch She'amar) on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/426?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H428" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/oAjWELNrN0I</t>
+          <t>https://youtu.be/nJQ_RbQIEvI</t>
         </is>
       </c>
       <c r="I428" s="2" t="n">
-        <v>221</v>
+        <v>200</v>
       </c>
       <c r="J428" s="2" t="n"/>
     </row>
@@ -18494,36 +18494,36 @@
       </c>
       <c r="C429" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D429" s="4" t="inlineStr">
         <is>
-          <t>רבי יהודה הנשיא</t>
+          <t>רבי נחמן קרוכמל (רנ״ק)</t>
         </is>
       </c>
       <c r="E429" s="7" t="inlineStr">
         <is>
-          <t>Рабби Йеуда ха-Наси: между завершением Мишны и руководством народом</t>
+          <t>Rabbi Nachman Krochmal (RaNaK) – The Thinker Who Turned History into Proof of the Eternity of Israel</t>
         </is>
       </c>
       <c r="F429" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/lik5L505iH0/edit</t>
+          <t>https://studio.youtube.com/video/oAjWELNrN0I/edit</t>
         </is>
       </c>
       <c r="G429" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Йехуда ха-Наси в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/580?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Nachman Krochmal (Ranak) on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/315?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H429" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/lik5L505iH0</t>
+          <t>https://youtu.be/oAjWELNrN0I</t>
         </is>
       </c>
       <c r="I429" s="2" t="n">
-        <v>358</v>
+        <v>221</v>
       </c>
       <c r="J429" s="2" t="n"/>
     </row>
@@ -18536,36 +18536,36 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D430" s="4" t="inlineStr">
         <is>
-          <t>רבי משה מקוצי (הסמ"ג)</t>
+          <t>רבי יהודה הנשיא</t>
         </is>
       </c>
       <c r="E430" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Moses of Coucy – the man who saw the Talmud burned and built a tower from it</t>
+          <t>Рабби Йеуда ха-Наси: между завершением Мишны и руководством народом</t>
         </is>
       </c>
       <c r="F430" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/diLTJBy2Jag/edit</t>
+          <t>https://studio.youtube.com/video/lik5L505iH0/edit</t>
         </is>
       </c>
       <c r="G430" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Moshe of Coucy (the Semag) on Ozar Chachamim — the full research and his teachers and students: https://ozar-chachamim-app.vercel.app/en/sage/588?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Йехуда ха-Наси в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/580?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H430" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/diLTJBy2Jag</t>
+          <t>https://youtu.be/lik5L505iH0</t>
         </is>
       </c>
       <c r="I430" s="2" t="n">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="J430" s="2" t="n"/>
     </row>
@@ -18578,36 +18578,36 @@
       </c>
       <c r="C431" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D431" s="4" t="inlineStr">
         <is>
-          <t>רבי יעקב אבן חביב (עין יעקב)</t>
+          <t>רבי משה מקוצי (הסמ"ג)</t>
         </is>
       </c>
       <c r="E431" s="7" t="inlineStr">
         <is>
-          <t>«Эйн Яаков»: мир и наследие рабби Яакова ибн Хабиба</t>
+          <t>Rabbi Moses of Coucy – the man who saw the Talmud burned and built a tower from it</t>
         </is>
       </c>
       <c r="F431" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/3RaB87PhVjs/edit</t>
+          <t>https://studio.youtube.com/video/diLTJBy2Jag/edit</t>
         </is>
       </c>
       <c r="G431" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Яаков ибн Хавив («Эйн Яаков») в «Оцар Хахамим» — полное исследование и его ученики: https://ozar-chachamim-app.vercel.app/ru/sage/603?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Moshe of Coucy (the Semag) on Ozar Chachamim — the full research and his teachers and students: https://ozar-chachamim-app.vercel.app/en/sage/588?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H431" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/3RaB87PhVjs</t>
+          <t>https://youtu.be/diLTJBy2Jag</t>
         </is>
       </c>
       <c r="I431" s="2" t="n">
-        <v>442</v>
+        <v>363</v>
       </c>
       <c r="J431" s="2" t="n"/>
     </row>
@@ -18625,31 +18625,31 @@
       </c>
       <c r="D432" s="4" t="inlineStr">
         <is>
-          <t>פרנץ רוזנצווייג – הפילוסוף שהחזיר את האדם למרכז</t>
+          <t>רבי יעקב אבן חביב (עין יעקב)</t>
         </is>
       </c>
       <c r="E432" s="7" t="inlineStr">
         <is>
-          <t>Франц Розенцвейг и его учение: иудейская теология и философия</t>
+          <t>«Эйн Яаков»: мир и наследие рабби Яакова ибн Хабиба</t>
         </is>
       </c>
       <c r="F432" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/fF1fkXyG-IU/edit</t>
+          <t>https://studio.youtube.com/video/3RaB87PhVjs/edit</t>
         </is>
       </c>
       <c r="G432" s="7" t="inlineStr">
         <is>
-          <t>📜 Франц Розенцвейг в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/141?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Яаков ибн Хавив («Эйн Яаков») в «Оцар Хахамим» — полное исследование и его ученики: https://ozar-chachamim-app.vercel.app/ru/sage/603?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H432" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/fF1fkXyG-IU</t>
+          <t>https://youtu.be/3RaB87PhVjs</t>
         </is>
       </c>
       <c r="I432" s="2" t="n">
-        <v>477</v>
+        <v>442</v>
       </c>
       <c r="J432" s="2" t="n"/>
     </row>
@@ -18662,36 +18662,36 @@
       </c>
       <c r="C433" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D433" s="4" t="inlineStr">
         <is>
-          <t>רבי מרדכי יפה – “בעל הלבוש”</t>
+          <t>פרנץ רוזנצווייג – הפילוסוף שהחזיר את האדם למרכז</t>
         </is>
       </c>
       <c r="E433" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Yaffe and the Architecture of the Golden Age</t>
+          <t>Франц Розенцвейг и его учение: иудейская теология и философия</t>
         </is>
       </c>
       <c r="F433" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/I4iSync7vvQ/edit</t>
+          <t>https://studio.youtube.com/video/fF1fkXyG-IU/edit</t>
         </is>
       </c>
       <c r="G433" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Mordechai Yaffe (the Ba'al ha-Levushim) on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/73?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Франц Розенцвейг в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/141?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H433" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/I4iSync7vvQ</t>
+          <t>https://youtu.be/fF1fkXyG-IU</t>
         </is>
       </c>
       <c r="I433" s="2" t="n">
-        <v>491</v>
+        <v>477</v>
       </c>
       <c r="J433" s="2" t="n"/>
     </row>
@@ -18709,31 +18709,31 @@
       </c>
       <c r="D434" s="4" t="inlineStr">
         <is>
-          <t>חכמי פרובנס – בין נרבון, בית דוד והמיסטיקה הראשונה: המרכז היהודי ששבר את המפה הרוחנית של ימי הביניים</t>
+          <t>רבי מרדכי יפה – “בעל הלבוש”</t>
         </is>
       </c>
       <c r="E434" s="7" t="inlineStr">
         <is>
-          <t>The Sages of Provence: Renaissance, Kabbalah, and Philosophy</t>
+          <t>Rabbi Yaffe and the Architecture of the Golden Age</t>
         </is>
       </c>
       <c r="F434" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/eGf4x9EmZPY/edit</t>
+          <t>https://studio.youtube.com/video/I4iSync7vvQ/edit</t>
         </is>
       </c>
       <c r="G434" s="7" t="inlineStr">
         <is>
-          <t>📜 The Sages of Provence on Ozar Chachamim — the page: https://ozar-chachamim-app.vercel.app/en/sage/38?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Mordechai Yaffe (the Ba'al ha-Levushim) on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/73?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H434" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/eGf4x9EmZPY</t>
+          <t>https://youtu.be/I4iSync7vvQ</t>
         </is>
       </c>
       <c r="I434" s="2" t="n">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="J434" s="2" t="n"/>
     </row>
@@ -18751,31 +18751,31 @@
       </c>
       <c r="D435" s="4" t="inlineStr">
         <is>
-          <t>רבי משה חגיז – הקנאי הירושלמי שניסה להציל את היהדות מן הקריסה הפנימית</t>
+          <t>חכמי פרובנס – בין נרבון, בית דוד והמיסטיקה הראשונה: המרכז היהודי ששבר את המפה הרוחנית של ימי הביניים</t>
         </is>
       </c>
       <c r="E435" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Moshe Hagiz – The Jerusalem Zealot Who Tried to Save Judaism from Internal Collapse</t>
+          <t>The Sages of Provence: Renaissance, Kabbalah, and Philosophy</t>
         </is>
       </c>
       <c r="F435" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/TBMI1NhMLYM/edit</t>
+          <t>https://studio.youtube.com/video/eGf4x9EmZPY/edit</t>
         </is>
       </c>
       <c r="G435" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Moshe Hagiz on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/86?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 The Sages of Provence on Ozar Chachamim — the page: https://ozar-chachamim-app.vercel.app/en/sage/38?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H435" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/TBMI1NhMLYM</t>
+          <t>https://youtu.be/eGf4x9EmZPY</t>
         </is>
       </c>
       <c r="I435" s="2" t="n">
-        <v>506</v>
+        <v>495</v>
       </c>
       <c r="J435" s="2" t="n"/>
     </row>
@@ -18793,31 +18793,31 @@
       </c>
       <c r="D436" s="4" t="inlineStr">
         <is>
-          <t>דונש בן לברט</t>
+          <t>רבי משה חגיז – הקנאי הירושלמי שניסה להציל את היהדות מן הקריסה הפנימית</t>
         </is>
       </c>
       <c r="E436" s="7" t="inlineStr">
         <is>
-          <t>Dunash ben Labrat: His Life and Works</t>
+          <t>Rabbi Moshe Hagiz – The Jerusalem Zealot Who Tried to Save Judaism from Internal Collapse</t>
         </is>
       </c>
       <c r="F436" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/Nh2zBFGV2_Q/edit</t>
+          <t>https://studio.youtube.com/video/TBMI1NhMLYM/edit</t>
         </is>
       </c>
       <c r="G436" s="7" t="inlineStr">
         <is>
-          <t>📜 Dunash ben Labrat on Ozar Chachamim — the full research, a quiz, and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/198?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Moshe Hagiz on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/86?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H436" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/Nh2zBFGV2_Q</t>
+          <t>https://youtu.be/TBMI1NhMLYM</t>
         </is>
       </c>
       <c r="I436" s="2" t="n">
-        <v>659</v>
+        <v>506</v>
       </c>
       <c r="J436" s="2" t="n"/>
     </row>
@@ -18830,36 +18830,36 @@
       </c>
       <c r="C437" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D437" s="4" t="inlineStr">
         <is>
-          <t>רבנו יונה גירונדי</t>
+          <t>דונש בן לברט</t>
         </is>
       </c>
       <c r="E437" s="7" t="inlineStr">
         <is>
-          <t>Рабейну Йона Гиронди: Тора, этика и полемика</t>
+          <t>Dunash ben Labrat: His Life and Works</t>
         </is>
       </c>
       <c r="F437" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/yCAH5_oIiX8/edit</t>
+          <t>https://studio.youtube.com/video/Nh2zBFGV2_Q/edit</t>
         </is>
       </c>
       <c r="G437" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабейну Йона Геронди в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/486?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Dunash ben Labrat on Ozar Chachamim — the full research, a quiz, and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/198?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H437" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/yCAH5_oIiX8</t>
+          <t>https://youtu.be/Nh2zBFGV2_Q</t>
         </is>
       </c>
       <c r="I437" s="2" t="n">
-        <v>703</v>
+        <v>659</v>
       </c>
       <c r="J437" s="2" t="n"/>
     </row>
@@ -18877,31 +18877,31 @@
       </c>
       <c r="D438" s="4" t="inlineStr">
         <is>
-          <t>הרב יצחק הוטנר</t>
+          <t>רבנו יונה גירונדי</t>
         </is>
       </c>
       <c r="E438" s="7" t="inlineStr">
         <is>
-          <t>Учение раввина Хутнера: «Пахад Ицхак» и «Даат»</t>
+          <t>Рабейну Йона Гиронди: Тора, этика и полемика</t>
         </is>
       </c>
       <c r="F438" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/vTYB_RodNy8/edit</t>
+          <t>https://studio.youtube.com/video/yCAH5_oIiX8/edit</t>
         </is>
       </c>
       <c r="G438" s="7" t="inlineStr">
         <is>
-          <t>📜 Рав Ицхак Хутнер в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/492?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабейну Йона Геронди в «Оцар Хахамим» — полное исследование, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/486?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H438" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/vTYB_RodNy8</t>
+          <t>https://youtu.be/yCAH5_oIiX8</t>
         </is>
       </c>
       <c r="I438" s="2" t="n">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="J438" s="2" t="n"/>
     </row>
@@ -18910,40 +18910,40 @@
         <v>438</v>
       </c>
       <c r="B439" s="3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C439" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D439" s="4" t="inlineStr">
         <is>
-          <t>רבי חנינא בר פפא</t>
+          <t>הרב יצחק הוטנר</t>
         </is>
       </c>
       <c r="E439" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Hanina bar Pappa - The Amora Who Asked the Angel of Death for 30 More Days</t>
+          <t>Учение раввина Хутнера: «Пахад Ицхак» и «Даат»</t>
         </is>
       </c>
       <c r="F439" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/xxmxesk4B6E/edit</t>
+          <t>https://studio.youtube.com/video/vTYB_RodNy8/edit</t>
         </is>
       </c>
       <c r="G439" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Chanina bar Pappa on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/543?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рав Ицхак Хутнер в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/492?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H439" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/xxmxesk4B6E</t>
+          <t>https://youtu.be/vTYB_RodNy8</t>
         </is>
       </c>
       <c r="I439" s="2" t="n">
-        <v>48</v>
+        <v>706</v>
       </c>
       <c r="J439" s="2" t="n"/>
     </row>
@@ -18956,36 +18956,36 @@
       </c>
       <c r="C440" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D440" s="4" t="inlineStr">
         <is>
-          <t>רבן שמעון בן גמליאל הראשון</t>
+          <t>רבי חנינא בר פפא</t>
         </is>
       </c>
       <c r="E440" s="7" t="inlineStr">
         <is>
-          <t>Раббан Шимон бен Гамлиэль I - Наси, пытавшийся спасти Иерусалим накануне разрушения</t>
+          <t>Rabbi Hanina bar Pappa - The Amora Who Asked the Angel of Death for 30 More Days</t>
         </is>
       </c>
       <c r="F440" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/lVKW3ot6R5E/edit</t>
+          <t>https://studio.youtube.com/video/xxmxesk4B6E/edit</t>
         </is>
       </c>
       <c r="G440" s="7" t="inlineStr">
         <is>
-          <t>📜 Раббан Шимон бен Гамлиэль Первый в «Оцар Хахамим» — полное исследование и его ученики: https://ozar-chachamim-app.vercel.app/ru/sage/550?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Chanina bar Pappa on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/543?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H440" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/lVKW3ot6R5E</t>
+          <t>https://youtu.be/xxmxesk4B6E</t>
         </is>
       </c>
       <c r="I440" s="2" t="n">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="J440" s="2" t="n"/>
     </row>
@@ -19003,31 +19003,31 @@
       </c>
       <c r="D441" s="4" t="inlineStr">
         <is>
-          <t>רבן יוחנן בן זכאי</t>
+          <t>רבן שמעון בן גמליאל הראשון</t>
         </is>
       </c>
       <c r="E441" s="7" t="inlineStr">
         <is>
-          <t>Раббан Йоханан бен Заккай: руководство народом и Тора в эпоху разрушения и восстановления</t>
+          <t>Раббан Шимон бен Гамлиэль I - Наси, пытавшийся спасти Иерусалим накануне разрушения</t>
         </is>
       </c>
       <c r="F441" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/PSlsgd30bzQ/edit</t>
+          <t>https://studio.youtube.com/video/lVKW3ot6R5E/edit</t>
         </is>
       </c>
       <c r="G441" s="7" t="inlineStr">
         <is>
-          <t>📜 Раббан Йоханан бен Заккай в «Оцар Хахамим» — полное исследование, викторина, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/592?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Раббан Шимон бен Гамлиэль Первый в «Оцар Хахамим» — полное исследование и его ученики: https://ozar-chachamim-app.vercel.app/ru/sage/550?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H441" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/PSlsgd30bzQ</t>
+          <t>https://youtu.be/lVKW3ot6R5E</t>
         </is>
       </c>
       <c r="I441" s="2" t="n">
-        <v>137</v>
+        <v>93</v>
       </c>
       <c r="J441" s="2" t="n"/>
     </row>
@@ -19040,36 +19040,36 @@
       </c>
       <c r="C442" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D442" s="4" t="inlineStr">
         <is>
-          <t>שרה אמנו</t>
+          <t>רבן יוחנן בן זכאי</t>
         </is>
       </c>
       <c r="E442" s="7" t="inlineStr">
         <is>
-          <t>Sarah Our Matriarch:The Foundation of Prophecy and the Sovereignty of Spirit in the Tent and in Time</t>
+          <t>Раббан Йоханан бен Заккай: руководство народом и Тора в эпоху разрушения и восстановления</t>
         </is>
       </c>
       <c r="F442" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/QHHa6EXkb8U/edit</t>
+          <t>https://studio.youtube.com/video/PSlsgd30bzQ/edit</t>
         </is>
       </c>
       <c r="G442" s="7" t="inlineStr">
         <is>
-          <t>📜 Sarah Our Matriarch on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/448?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Раббан Йоханан бен Заккай в «Оцар Хахамим» — полное исследование, викторина, а также его учителя и ученики: https://ozar-chachamim-app.vercel.app/ru/sage/592?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H442" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/QHHa6EXkb8U</t>
+          <t>https://youtu.be/PSlsgd30bzQ</t>
         </is>
       </c>
       <c r="I442" s="2" t="n">
-        <v>179</v>
+        <v>137</v>
       </c>
       <c r="J442" s="2" t="n"/>
     </row>
@@ -19885,31 +19885,31 @@
       </c>
       <c r="D462" s="4" t="inlineStr">
         <is>
-          <t>הרב כלפון משה הכהן (1874–1950) – רב ג'רבא: הלכה, הנהגה וציונות דתית בצפון אפריקה</t>
+          <t>הרב נתן צבי פינקל (הסבא מסלבודקה)</t>
         </is>
       </c>
       <c r="E462" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Khalfon: Halakhic Decisor and Zionist Leader</t>
+          <t>The Grandfather of Slabodka and the Kingdom of Human Greatness: From Lithuania to Hebron &amp; Jerusalem</t>
         </is>
       </c>
       <c r="F462" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/rrilooQ8bSw/edit</t>
+          <t>https://studio.youtube.com/video/XqiW1-Q_dkY/edit</t>
         </is>
       </c>
       <c r="G462" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Khalfon Moshe HaKohen on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/136?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Nosson Tzvi Finkel (the Alter of Slabodka) on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/324?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H462" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/rrilooQ8bSw</t>
+          <t>https://youtu.be/XqiW1-Q_dkY</t>
         </is>
       </c>
       <c r="I462" s="2" t="n">
-        <v>538</v>
+        <v>341</v>
       </c>
       <c r="J462" s="2" t="n"/>
     </row>
@@ -19927,31 +19927,31 @@
       </c>
       <c r="D463" s="4" t="inlineStr">
         <is>
-          <t>הרב מאיר זייני</t>
+          <t>הרב כלפון משה הכהן (1874–1950) – רב ג'רבא: הלכה, הנהגה וציונות דתית בצפון אפריקה</t>
         </is>
       </c>
       <c r="E463" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Meir Zini: The Heroic Leader Bridging Algeria, Auschwitz, and Montmartre</t>
+          <t>Rabbi Khalfon: Halakhic Decisor and Zionist Leader</t>
         </is>
       </c>
       <c r="F463" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/TRDE4AG2kLE/edit</t>
+          <t>https://studio.youtube.com/video/rrilooQ8bSw/edit</t>
         </is>
       </c>
       <c r="G463" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Meir Zeini on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/165?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Khalfon Moshe HaKohen on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/136?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H463" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/TRDE4AG2kLE</t>
+          <t>https://youtu.be/rrilooQ8bSw</t>
         </is>
       </c>
       <c r="I463" s="2" t="n">
-        <v>597</v>
+        <v>538</v>
       </c>
       <c r="J463" s="2" t="n"/>
     </row>
@@ -19964,36 +19964,36 @@
       </c>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D464" s="4" t="inlineStr">
         <is>
-          <t>רבי רפאל משה לוריא</t>
+          <t>הרב מאיר זייני</t>
         </is>
       </c>
       <c r="E464" s="7" t="inlineStr">
         <is>
-          <t>Раввин Моше Лурия: каббалист и учёный</t>
+          <t>Rabbi Meir Zini: The Heroic Leader Bridging Algeria, Auschwitz, and Montmartre</t>
         </is>
       </c>
       <c r="F464" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/OvfCDsr2-p4/edit</t>
+          <t>https://studio.youtube.com/video/TRDE4AG2kLE/edit</t>
         </is>
       </c>
       <c r="G464" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Рефаэль Моше Лурия в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/174?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Meir Zeini on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/165?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H464" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/OvfCDsr2-p4</t>
+          <t>https://youtu.be/TRDE4AG2kLE</t>
         </is>
       </c>
       <c r="I464" s="2" t="n">
-        <v>621</v>
+        <v>597</v>
       </c>
       <c r="J464" s="2" t="n"/>
     </row>
@@ -20006,36 +20006,36 @@
       </c>
       <c r="C465" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D465" s="4" t="inlineStr">
         <is>
-          <t>רבי יוסף טאיטצאק – המקובל שחזה את הציונות</t>
+          <t>רבי רפאל משה לוריא</t>
         </is>
       </c>
       <c r="E465" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Yosef Taitatzak - The Kabbalist Who Foresaw Zionism</t>
+          <t>Раввин Моше Лурия: каббалист и учёный</t>
         </is>
       </c>
       <c r="F465" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/sCJ-e_Ggy68/edit</t>
+          <t>https://studio.youtube.com/video/OvfCDsr2-p4/edit</t>
         </is>
       </c>
       <c r="G465" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Yosef Taitazak on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/68?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Рефаэль Моше Лурия в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/174?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H465" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/sCJ-e_Ggy68</t>
+          <t>https://youtu.be/OvfCDsr2-p4</t>
         </is>
       </c>
       <c r="I465" s="2" t="n">
-        <v>673</v>
+        <v>621</v>
       </c>
       <c r="J465" s="2" t="n"/>
     </row>
@@ -20048,36 +20048,36 @@
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>עברית</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D466" s="4" t="inlineStr">
         <is>
-          <t>חכם דוד ניטו</t>
-        </is>
-      </c>
-      <c r="E466" s="5" t="inlineStr">
-        <is>
-          <t>דוד ניטו: מטה דן ופולמוס הטבע</t>
+          <t>רבי יוסף טאיטצאק – המקובל שחזה את הציונות</t>
+        </is>
+      </c>
+      <c r="E466" s="7" t="inlineStr">
+        <is>
+          <t>Rabbi Yosef Taitatzak - The Kabbalist Who Foresaw Zionism</t>
         </is>
       </c>
       <c r="F466" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/dT4vX4G3LJk/edit</t>
-        </is>
-      </c>
-      <c r="G466" s="5" t="inlineStr">
-        <is>
-          <t>📜 חכם דוד ניטו באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/487?utm_source=youtube&amp;utm_medium=video</t>
+          <t>https://studio.youtube.com/video/sCJ-e_Ggy68/edit</t>
+        </is>
+      </c>
+      <c r="G466" s="7" t="inlineStr">
+        <is>
+          <t>📜 Rabbi Yosef Taitazak on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/68?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H466" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/dT4vX4G3LJk</t>
+          <t>https://youtu.be/sCJ-e_Ggy68</t>
         </is>
       </c>
       <c r="I466" s="2" t="n">
-        <v>729</v>
+        <v>673</v>
       </c>
       <c r="J466" s="2" t="n"/>
     </row>
@@ -20086,40 +20086,40 @@
         <v>466</v>
       </c>
       <c r="B467" s="3" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C467" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>עברית</t>
         </is>
       </c>
       <c r="D467" s="4" t="inlineStr">
         <is>
-          <t>רבי אברהם בן שלמה הלוי בוקראט</t>
-        </is>
-      </c>
-      <c r="E467" s="7" t="inlineStr">
-        <is>
-          <t>Rabbi Abraham Bokrat - The Scholar Expelled from Spain Who Rose to Rashi’s Defense</t>
+          <t>חכם דוד ניטו</t>
+        </is>
+      </c>
+      <c r="E467" s="5" t="inlineStr">
+        <is>
+          <t>דוד ניטו: מטה דן ופולמוס הטבע</t>
         </is>
       </c>
       <c r="F467" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/3tqZnY6xxJ4/edit</t>
-        </is>
-      </c>
-      <c r="G467" s="7" t="inlineStr">
-        <is>
-          <t>📜 Rabbi Abraham ben Solomon HaLevi Bokrat on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/627?utm_source=youtube&amp;utm_medium=video</t>
+          <t>https://studio.youtube.com/video/dT4vX4G3LJk/edit</t>
+        </is>
+      </c>
+      <c r="G467" s="5" t="inlineStr">
+        <is>
+          <t>📜 חכם דוד ניטו באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/487?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H467" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/3tqZnY6xxJ4</t>
+          <t>https://youtu.be/dT4vX4G3LJk</t>
         </is>
       </c>
       <c r="I467" s="2" t="n">
-        <v>8</v>
+        <v>729</v>
       </c>
       <c r="J467" s="2" t="n"/>
     </row>
@@ -20137,31 +20137,31 @@
       </c>
       <c r="D468" s="4" t="inlineStr">
         <is>
-          <t>הרבנית אסתר יונגרייז</t>
+          <t>רבי אברהם בן שלמה הלוי בוקראט</t>
         </is>
       </c>
       <c r="E468" s="7" t="inlineStr">
         <is>
-          <t>A Call from the Ashes: The Legacy of Rebbetzin Esther Jungreis and the Hineni Movement</t>
+          <t>Rabbi Abraham Bokrat - The Scholar Expelled from Spain Who Rose to Rashi’s Defense</t>
         </is>
       </c>
       <c r="F468" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/qr-Jzk95mEA/edit</t>
+          <t>https://studio.youtube.com/video/3tqZnY6xxJ4/edit</t>
         </is>
       </c>
       <c r="G468" s="7" t="inlineStr">
         <is>
-          <t>📜 Rebbetzin Esther Jungreis on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/514?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Abraham ben Solomon HaLevi Bokrat on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/627?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H468" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/qr-Jzk95mEA</t>
+          <t>https://youtu.be/3tqZnY6xxJ4</t>
         </is>
       </c>
       <c r="I468" s="2" t="n">
-        <v>115</v>
+        <v>8</v>
       </c>
       <c r="J468" s="2" t="n"/>
     </row>
@@ -20179,31 +20179,31 @@
       </c>
       <c r="D469" s="4" t="inlineStr">
         <is>
-          <t>שמאי הזקן</t>
+          <t>הרבנית אסתר יונגרייז</t>
         </is>
       </c>
       <c r="E469" s="7" t="inlineStr">
         <is>
-          <t>Shammai the Elder: His Character, Teachings, and the Legacy of the House of Shammai</t>
+          <t>A Call from the Ashes: The Legacy of Rebbetzin Esther Jungreis and the Hineni Movement</t>
         </is>
       </c>
       <c r="F469" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/TuIOTBpjNZE/edit</t>
+          <t>https://studio.youtube.com/video/qr-Jzk95mEA/edit</t>
         </is>
       </c>
       <c r="G469" s="7" t="inlineStr">
         <is>
-          <t>📜 Shammai the Elder on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/504?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rebbetzin Esther Jungreis on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/514?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H469" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/TuIOTBpjNZE</t>
+          <t>https://youtu.be/qr-Jzk95mEA</t>
         </is>
       </c>
       <c r="I469" s="2" t="n">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="J469" s="2" t="n"/>
     </row>
@@ -20216,36 +20216,36 @@
       </c>
       <c r="C470" s="2" t="inlineStr">
         <is>
-          <t>Русский</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D470" s="4" t="inlineStr">
         <is>
-          <t>רבינו דוד בונפיד</t>
+          <t>שמאי הזקן</t>
         </is>
       </c>
       <c r="E470" s="7" t="inlineStr">
         <is>
-          <t>Рав Давид Бонафед: ученик Рамбана и его духовное наследие в Испании</t>
+          <t>Shammai the Elder: His Character, Teachings, and the Legacy of the House of Shammai</t>
         </is>
       </c>
       <c r="F470" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/pGDFGE42KoM/edit</t>
+          <t>https://studio.youtube.com/video/TuIOTBpjNZE/edit</t>
         </is>
       </c>
       <c r="G470" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабейну Давид Бонафед в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/460?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Shammai the Elder on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/504?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H470" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/pGDFGE42KoM</t>
+          <t>https://youtu.be/TuIOTBpjNZE</t>
         </is>
       </c>
       <c r="I470" s="2" t="n">
-        <v>167</v>
+        <v>132</v>
       </c>
       <c r="J470" s="2" t="n"/>
     </row>
@@ -20263,31 +20263,31 @@
       </c>
       <c r="D471" s="4" t="inlineStr">
         <is>
-          <t>רבי סעדיה שוראקי</t>
+          <t>רבינו דוד בונפיד</t>
         </is>
       </c>
       <c r="E471" s="7" t="inlineStr">
         <is>
-          <t>Рабби Саадия Шураки — раввин, который ввёл математику в дом учения</t>
+          <t>Рав Давид Бонафед: ученик Рамбана и его духовное наследие в Испании</t>
         </is>
       </c>
       <c r="F471" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/ZY7m_A8SBuA/edit</t>
+          <t>https://studio.youtube.com/video/pGDFGE42KoM/edit</t>
         </is>
       </c>
       <c r="G471" s="7" t="inlineStr">
         <is>
-          <t>📜 Рабби Саадья Шураки в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/277?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабейну Давид Бонафед в «Оцар Хахамим» — полное исследование и его учителя: https://ozar-chachamim-app.vercel.app/ru/sage/460?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H471" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/ZY7m_A8SBuA</t>
+          <t>https://youtu.be/pGDFGE42KoM</t>
         </is>
       </c>
       <c r="I471" s="2" t="n">
-        <v>269</v>
+        <v>167</v>
       </c>
       <c r="J471" s="2" t="n"/>
     </row>
@@ -20300,36 +20300,36 @@
       </c>
       <c r="C472" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Русский</t>
         </is>
       </c>
       <c r="D472" s="4" t="inlineStr">
         <is>
-          <t>רבי משה הדרשן</t>
+          <t>רבי סעדיה שוראקי</t>
         </is>
       </c>
       <c r="E472" s="7" t="inlineStr">
         <is>
-          <t>Rabbi Moshe HaDarshan – The Sage Who Shaped the World of Midrash in Europe</t>
+          <t>Рабби Саадия Шураки — раввин, который ввёл математику в дом учения</t>
         </is>
       </c>
       <c r="F472" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/B7dQL1mV29k/edit</t>
+          <t>https://studio.youtube.com/video/ZY7m_A8SBuA/edit</t>
         </is>
       </c>
       <c r="G472" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Moshe HaDarshan on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/348?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Рабби Саадья Шураки в «Оцар Хахамим» — полное исследование: https://ozar-chachamim-app.vercel.app/ru/sage/277?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H472" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/B7dQL1mV29k</t>
+          <t>https://youtu.be/ZY7m_A8SBuA</t>
         </is>
       </c>
       <c r="I472" s="2" t="n">
-        <v>302</v>
+        <v>269</v>
       </c>
       <c r="J472" s="2" t="n"/>
     </row>
@@ -20347,31 +20347,31 @@
       </c>
       <c r="D473" s="4" t="inlineStr">
         <is>
-          <t>רבי דוד פארדו</t>
+          <t>רבי משה הדרשן</t>
         </is>
       </c>
       <c r="E473" s="7" t="inlineStr">
         <is>
-          <t>Rabbi David Pardo and the Revolution in Tosefta Interpretation in Chasdei David</t>
+          <t>Rabbi Moshe HaDarshan – The Sage Who Shaped the World of Midrash in Europe</t>
         </is>
       </c>
       <c r="F473" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/U6Jz3o9QeI0/edit</t>
+          <t>https://studio.youtube.com/video/B7dQL1mV29k/edit</t>
         </is>
       </c>
       <c r="G473" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi David Pardo on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/349?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi Moshe HaDarshan on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/348?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H473" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/U6Jz3o9QeI0</t>
+          <t>https://youtu.be/B7dQL1mV29k</t>
         </is>
       </c>
       <c r="I473" s="2" t="n">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="J473" s="2" t="n"/>
     </row>
@@ -20389,31 +20389,31 @@
       </c>
       <c r="D474" s="4" t="inlineStr">
         <is>
-          <t>רבנו בחיי בן אשר</t>
+          <t>רבי דוד פארדו</t>
         </is>
       </c>
       <c r="E474" s="7" t="inlineStr">
         <is>
-          <t>Rabbeinu  Bahya ben Asher: Between Peshat and Sod</t>
+          <t>Rabbi David Pardo and the Revolution in Tosefta Interpretation in Chasdei David</t>
         </is>
       </c>
       <c r="F474" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/A9WGoajqE-g/edit</t>
+          <t>https://studio.youtube.com/video/U6Jz3o9QeI0/edit</t>
         </is>
       </c>
       <c r="G474" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbenu Bachya ben Asher on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/12?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbi David Pardo on Ozar Chachamim — the full research: https://ozar-chachamim-app.vercel.app/en/sage/349?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H474" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/A9WGoajqE-g</t>
+          <t>https://youtu.be/U6Jz3o9QeI0</t>
         </is>
       </c>
       <c r="I474" s="2" t="n">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="J474" s="2" t="n"/>
     </row>
@@ -20431,31 +20431,31 @@
       </c>
       <c r="D475" s="4" t="inlineStr">
         <is>
-          <t>הרב נתן צבי פינקל (הסבא מסלבודקה)</t>
+          <t>רבנו בחיי בן אשר</t>
         </is>
       </c>
       <c r="E475" s="7" t="inlineStr">
         <is>
-          <t>The Grandfather of Slabodka and the Kingdom of Human Greatness: From Lithuania to Hebron &amp; Jerusalem</t>
+          <t>Rabbeinu  Bahya ben Asher: Between Peshat and Sod</t>
         </is>
       </c>
       <c r="F475" s="6" t="inlineStr">
         <is>
-          <t>https://studio.youtube.com/video/XqiW1-Q_dkY/edit</t>
+          <t>https://studio.youtube.com/video/A9WGoajqE-g/edit</t>
         </is>
       </c>
       <c r="G475" s="7" t="inlineStr">
         <is>
-          <t>📜 Rabbi Nosson Tzvi Finkel (the Alter of Slabodka) on Ozar Chachamim — the full research and his students: https://ozar-chachamim-app.vercel.app/en/sage/324?utm_source=youtube&amp;utm_medium=video</t>
+          <t>📜 Rabbenu Bachya ben Asher on Ozar Chachamim — the full research and his teachers: https://ozar-chachamim-app.vercel.app/en/sage/12?utm_source=youtube&amp;utm_medium=video</t>
         </is>
       </c>
       <c r="H475" s="6" t="inlineStr">
         <is>
-          <t>https://youtu.be/XqiW1-Q_dkY</t>
+          <t>https://youtu.be/A9WGoajqE-g</t>
         </is>
       </c>
       <c r="I475" s="2" t="n">
-        <v>341</v>
+        <v>313</v>
       </c>
       <c r="J475" s="2" t="n"/>
     </row>
@@ -32491,7 +32491,7 @@
         </is>
       </c>
       <c r="E2" s="3" t="n">
-        <v>1885</v>
+        <v>1890</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>148</v>
@@ -32680,7 +32680,7 @@
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>129</v>
@@ -32923,7 +32923,7 @@
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>192</v>
@@ -33139,7 +33139,7 @@
         </is>
       </c>
       <c r="E26" s="3" t="n">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>151</v>
@@ -33868,7 +33868,7 @@
         </is>
       </c>
       <c r="E53" s="3" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F53" s="2" t="n">
         <v>631</v>
@@ -34057,7 +34057,7 @@
         </is>
       </c>
       <c r="E60" s="3" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F60" s="2" t="n">
         <v>108</v>
@@ -34300,7 +34300,7 @@
         </is>
       </c>
       <c r="E69" s="3" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F69" s="2" t="n">
         <v>17</v>
@@ -34624,7 +34624,7 @@
         </is>
       </c>
       <c r="E81" s="3" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F81" s="2" t="n">
         <v>180</v>
@@ -34853,24 +34853,24 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>יעקב בן אשר</t>
+          <t>אליהו בן אמוזג – ההוגה שדחו הדורות, אך רעיונו התגלה כגדול מדורותיו</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/1ascElHzBKieDVSWk8wZBw</t>
+          <t>https://open.spotify.com/episode/66ocgEWzF0dAp3RmcvYSAn</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>📜 יעקב בן אשר באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/189?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 אליהו בן אמוזג באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/118?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E90" s="3" t="n">
         <v>145</v>
       </c>
       <c r="F90" s="2" t="n">
-        <v>189</v>
+        <v>118</v>
       </c>
       <c r="G90" s="2" t="n"/>
     </row>
@@ -34880,24 +34880,24 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>רבי יוסף חיון (רי״ח)</t>
+          <t>יעקב בן אשר</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/5J3m8GmCr0dbgQl0IyUyW6</t>
+          <t>https://open.spotify.com/episode/1ascElHzBKieDVSWk8wZBw</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי יוסף חיון (רי״ח) באוצר חכמים — המחקר המלא ורבותיו ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/19?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 יעקב בן אשר באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/189?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E91" s="3" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>19</v>
+        <v>189</v>
       </c>
       <c r="G91" s="2" t="n"/>
     </row>
@@ -34907,24 +34907,24 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>אליהו בן אמוזג – ההוגה שדחו הדורות, אך רעיונו התגלה כגדול מדורותיו</t>
+          <t>רבי יוסף חיון (רי״ח)</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/66ocgEWzF0dAp3RmcvYSAn</t>
+          <t>https://open.spotify.com/episode/5J3m8GmCr0dbgQl0IyUyW6</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>📜 אליהו בן אמוזג באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/118?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי יוסף חיון (רי״ח) באוצר חכמים — המחקר המלא ורבותיו ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/19?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E92" s="3" t="n">
         <v>144</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>118</v>
+        <v>19</v>
       </c>
       <c r="G92" s="2" t="n"/>
     </row>
@@ -35299,7 +35299,7 @@
         </is>
       </c>
       <c r="E106" s="3" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F106" s="2" t="n">
         <v>154</v>
@@ -35312,24 +35312,24 @@
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>רבי שם טוב אבן גאון</t>
+          <t>פרנץ רוזנצווייג – הפילוסוף שהחזיר את האדם למרכז</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/4WLBwaZKgmiVJPIACa5dJR</t>
+          <t>https://open.spotify.com/episode/7EpaIjYgIJVmSWDAsXDI7g</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי שם טוב אבן גאון באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/415?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 פרנץ רוזנצווייג באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/141?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E107" s="3" t="n">
         <v>120</v>
       </c>
       <c r="F107" s="2" t="n">
-        <v>415</v>
+        <v>141</v>
       </c>
       <c r="G107" s="2" t="n"/>
     </row>
@@ -35339,24 +35339,24 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>האדמו"ר מפיאסצ'נה (1889–1942) – קודש בתוך החורבן: תורה פסיכולוגית, אמונה ועמידה בגטו ורשה</t>
+          <t>רבי שם טוב אבן גאון</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/462p60k0hrJUeoi1OiEtfD</t>
+          <t>https://open.spotify.com/episode/4WLBwaZKgmiVJPIACa5dJR</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>📜 האדמו״ר מפיאסצ׳נה באוצר חכמים — המחקר המלא וחידון: https://ozar-chachamim-app.vercel.app/he/sage/143?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי שם טוב אבן גאון באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/415?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E108" s="3" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F108" s="2" t="n">
-        <v>143</v>
+        <v>415</v>
       </c>
       <c r="G108" s="2" t="n"/>
     </row>
@@ -35366,24 +35366,24 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>אברהם בר חייא</t>
+          <t>האדמו"ר מפיאסצ'נה (1889–1942) – קודש בתוך החורבן: תורה פסיכולוגית, אמונה ועמידה בגטו ורשה</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/3FAGqYdzyMQbyPbon3KYoC</t>
+          <t>https://open.spotify.com/episode/462p60k0hrJUeoi1OiEtfD</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>📜 אברהם בר חייא באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/190?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 האדמו״ר מפיאסצ׳נה באוצר חכמים — המחקר המלא וחידון: https://ozar-chachamim-app.vercel.app/he/sage/143?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E109" s="3" t="n">
         <v>118</v>
       </c>
       <c r="F109" s="2" t="n">
-        <v>190</v>
+        <v>143</v>
       </c>
       <c r="G109" s="2" t="n"/>
     </row>
@@ -35393,24 +35393,24 @@
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>רבי חנינא בר פפא</t>
+          <t>אברהם בר חייא</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/05UPnPXXJ2u149d7DKjKzG</t>
+          <t>https://open.spotify.com/episode/3FAGqYdzyMQbyPbon3KYoC</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי חנינא בר פפא באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/543?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 אברהם בר חייא באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/190?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E110" s="3" t="n">
         <v>118</v>
       </c>
       <c r="F110" s="2" t="n">
-        <v>543</v>
+        <v>190</v>
       </c>
       <c r="G110" s="2" t="n"/>
     </row>
@@ -35420,24 +35420,24 @@
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>רבי משה חיים לוצאטו (הרמח״ל)</t>
+          <t>רבי חנינא בר פפא</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/1lgKTjkSyrd7SAntCbBGTt</t>
+          <t>https://open.spotify.com/episode/05UPnPXXJ2u149d7DKjKzG</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי משה חיים לוצאטו (הרמח״ל) באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/93?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי חנינא בר פפא באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/543?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E111" s="3" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F111" s="2" t="n">
-        <v>93</v>
+        <v>543</v>
       </c>
       <c r="G111" s="2" t="n"/>
     </row>
@@ -35447,24 +35447,24 @@
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>שמעון כיפא – מרטיר נוצרי או צדיק נסתר ששלחו חכמי ישראל?</t>
+          <t>רבי משה חיים לוצאטו (הרמח״ל)</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/4tu43oeL4qVdXGKzX2025J</t>
+          <t>https://open.spotify.com/episode/1lgKTjkSyrd7SAntCbBGTt</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
         <is>
-          <t>📜 שמעון כיפא באוצר חכמים — הדף שלו: https://ozar-chachamim-app.vercel.app/he/sage/193?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי משה חיים לוצאטו (הרמח״ל) באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/93?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E112" s="3" t="n">
         <v>117</v>
       </c>
       <c r="F112" s="2" t="n">
-        <v>193</v>
+        <v>93</v>
       </c>
       <c r="G112" s="2" t="n"/>
     </row>
@@ -35474,24 +35474,24 @@
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>פרנץ רוזנצווייג – הפילוסוף שהחזיר את האדם למרכז</t>
+          <t>שמעון כיפא – מרטיר נוצרי או צדיק נסתר ששלחו חכמי ישראל?</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/7EpaIjYgIJVmSWDAsXDI7g</t>
+          <t>https://open.spotify.com/episode/4tu43oeL4qVdXGKzX2025J</t>
         </is>
       </c>
       <c r="D113" s="5" t="inlineStr">
         <is>
-          <t>📜 פרנץ רוזנצווייג באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/141?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 שמעון כיפא באוצר חכמים — הדף שלו: https://ozar-chachamim-app.vercel.app/he/sage/193?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E113" s="3" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F113" s="2" t="n">
-        <v>141</v>
+        <v>193</v>
       </c>
       <c r="G113" s="2" t="n"/>
     </row>
@@ -35555,24 +35555,24 @@
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>רבי יחיאל מפריז</t>
+          <t>ילקוט שמעוני</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/46MHn4vu6ORF3S4hyf9rN9</t>
+          <t>https://open.spotify.com/episode/7tKvMKCTFSZebvK2vj0U5b</t>
         </is>
       </c>
       <c r="D116" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי יחיאל מפריז באוצר חכמים — המחקר המלא ורבותיו ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/54?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 ילקוט שמעוני באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/55?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E116" s="3" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F116" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G116" s="2" t="n"/>
     </row>
@@ -35582,24 +35582,24 @@
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>ילקוט שמעוני</t>
+          <t>רבי יחיאל מפריז</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/7tKvMKCTFSZebvK2vj0U5b</t>
+          <t>https://open.spotify.com/episode/46MHn4vu6ORF3S4hyf9rN9</t>
         </is>
       </c>
       <c r="D117" s="5" t="inlineStr">
         <is>
-          <t>📜 ילקוט שמעוני באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/55?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי יחיאל מפריז באוצר חכמים — המחקר המלא ורבותיו ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/54?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E117" s="3" t="n">
         <v>111</v>
       </c>
       <c r="F117" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G117" s="2" t="n"/>
     </row>
@@ -36149,24 +36149,24 @@
       </c>
       <c r="B138" s="4" t="inlineStr">
         <is>
-          <t>רבי שמשון בן צדוק</t>
+          <t>הרב שמואל בורנשטיין – בעל 'שם משמואל'</t>
         </is>
       </c>
       <c r="C138" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/5icFLQJoUIWSCfgYau1reF</t>
+          <t>https://open.spotify.com/episode/5dTIktS4k7pzb2kSQbqtXB</t>
         </is>
       </c>
       <c r="D138" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי שמשון בן צדוק באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/317?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 הרב שמואל בורנשטיין באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/131?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E138" s="3" t="n">
         <v>94</v>
       </c>
       <c r="F138" s="2" t="n">
-        <v>317</v>
+        <v>131</v>
       </c>
       <c r="G138" s="2" t="n"/>
     </row>
@@ -36176,24 +36176,24 @@
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>רבנו תם (ר׳ יעקב בן מאיר) – מהפכן השיטה התוספתית</t>
+          <t>רבי שמשון בן צדוק</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/5u9zxyAssijvwzZnbKM7OQ</t>
+          <t>https://open.spotify.com/episode/5icFLQJoUIWSCfgYau1reF</t>
         </is>
       </c>
       <c r="D139" s="5" t="inlineStr">
         <is>
-          <t>📜 רבנו תם (ר׳ יעקב בן מאיר) באוצר חכמים — המחקר המלא ורבותיו ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/33?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי שמשון בן צדוק באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/317?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E139" s="3" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F139" s="2" t="n">
-        <v>33</v>
+        <v>317</v>
       </c>
       <c r="G139" s="2" t="n"/>
     </row>
@@ -36203,24 +36203,24 @@
       </c>
       <c r="B140" s="4" t="inlineStr">
         <is>
-          <t>רבי יצחק סגי נהור</t>
+          <t>רבנו תם (ר׳ יעקב בן מאיר) – מהפכן השיטה התוספתית</t>
         </is>
       </c>
       <c r="C140" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/16NM4luayYQvcaoGO21kWg</t>
+          <t>https://open.spotify.com/episode/5u9zxyAssijvwzZnbKM7OQ</t>
         </is>
       </c>
       <c r="D140" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי יצחק סגי נהור באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/42?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבנו תם (ר׳ יעקב בן מאיר) באוצר חכמים — המחקר המלא ורבותיו ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/33?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E140" s="3" t="n">
         <v>93</v>
       </c>
       <c r="F140" s="2" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="G140" s="2" t="n"/>
     </row>
@@ -36230,24 +36230,24 @@
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>הרב שמואל בורנשטיין – בעל 'שם משמואל'</t>
+          <t>רבי יצחק סגי נהור</t>
         </is>
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/5dTIktS4k7pzb2kSQbqtXB</t>
+          <t>https://open.spotify.com/episode/16NM4luayYQvcaoGO21kWg</t>
         </is>
       </c>
       <c r="D141" s="5" t="inlineStr">
         <is>
-          <t>📜 הרב שמואל בורנשטיין באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/131?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי יצחק סגי נהור באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/42?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E141" s="3" t="n">
         <v>93</v>
       </c>
       <c r="F141" s="2" t="n">
-        <v>131</v>
+        <v>42</v>
       </c>
       <c r="G141" s="2" t="n"/>
     </row>
@@ -36608,24 +36608,24 @@
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>תודוס איש רומי</t>
+          <t>רבי אלעזר מגרמייזא (בעל הרוקח)</t>
         </is>
       </c>
       <c r="C155" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/5FpiW245vsxYv7x3SXzLgq</t>
+          <t>https://open.spotify.com/episode/1xnTTOc3bgPDd10LUBerVb</t>
         </is>
       </c>
       <c r="D155" s="5" t="inlineStr">
         <is>
-          <t>📜 תודוס איש רומי באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/485?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי אלעזר מגרמייזא (בעל הרוקח) באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/280?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E155" s="3" t="n">
         <v>78</v>
       </c>
       <c r="F155" s="2" t="n">
-        <v>485</v>
+        <v>280</v>
       </c>
       <c r="G155" s="2" t="n"/>
     </row>
@@ -36635,24 +36635,24 @@
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>רבי יהודה החסיד (חסידי אשכנז)</t>
+          <t>תודוס איש רומי</t>
         </is>
       </c>
       <c r="C156" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/70SOBeANLpCEBeEplD3eOw</t>
+          <t>https://open.spotify.com/episode/5FpiW245vsxYv7x3SXzLgq</t>
         </is>
       </c>
       <c r="D156" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי יהודה החסיד (חסידי אשכנז) באוצר חכמים — המחקר המלא ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/11?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 תודוס איש רומי באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/485?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E156" s="3" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F156" s="2" t="n">
-        <v>11</v>
+        <v>485</v>
       </c>
       <c r="G156" s="2" t="n"/>
     </row>
@@ -36662,24 +36662,24 @@
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>רבי אפרים אנקווה – 'הרב הרוכב על האריה'</t>
+          <t>רבי יהודה החסיד (חסידי אשכנז)</t>
         </is>
       </c>
       <c r="C157" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/7q3U1w91U94YzhWhEWkgSB</t>
+          <t>https://open.spotify.com/episode/70SOBeANLpCEBeEplD3eOw</t>
         </is>
       </c>
       <c r="D157" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי אפרים אנקווה באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/58?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי יהודה החסיד (חסידי אשכנז) באוצר חכמים — המחקר המלא ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/11?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E157" s="3" t="n">
         <v>77</v>
       </c>
       <c r="F157" s="2" t="n">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="G157" s="2" t="n"/>
     </row>
@@ -36689,24 +36689,24 @@
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>רבי אלעזר מגרמייזא (בעל הרוקח)</t>
+          <t>רבי אפרים אנקווה – 'הרב הרוכב על האריה'</t>
         </is>
       </c>
       <c r="C158" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/1xnTTOc3bgPDd10LUBerVb</t>
+          <t>https://open.spotify.com/episode/7q3U1w91U94YzhWhEWkgSB</t>
         </is>
       </c>
       <c r="D158" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי אלעזר מגרמייזא (בעל הרוקח) באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/280?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי אפרים אנקווה באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/58?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E158" s="3" t="n">
         <v>77</v>
       </c>
       <c r="F158" s="2" t="n">
-        <v>280</v>
+        <v>58</v>
       </c>
       <c r="G158" s="2" t="n"/>
     </row>
@@ -38795,24 +38795,24 @@
       </c>
       <c r="B236" s="4" t="inlineStr">
         <is>
-          <t>רבי אלעזר בן עזריה</t>
+          <t>הרב נתן צבי פינקל (הסבא מסלבודקה)</t>
         </is>
       </c>
       <c r="C236" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/581Qie3gJwcdnadi7wnNF2</t>
+          <t>https://open.spotify.com/episode/4iRZ0WdzCGhxJrGTmkAzUf</t>
         </is>
       </c>
       <c r="D236" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי אלעזר בן עזריה באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/506?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 הרב נתן צבי פינקל (הסבא מסלבודקה) באוצר חכמים — המחקר המלא ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/324?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E236" s="3" t="n">
         <v>44</v>
       </c>
       <c r="F236" s="2" t="n">
-        <v>506</v>
+        <v>324</v>
       </c>
       <c r="G236" s="2" t="n"/>
     </row>
@@ -38822,24 +38822,24 @@
       </c>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t>רבי שמעון לביא</t>
+          <t>רבי אלעזר בן עזריה</t>
         </is>
       </c>
       <c r="C237" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/09sbxccxPcM8mqxUj6yDR4</t>
+          <t>https://open.spotify.com/episode/581Qie3gJwcdnadi7wnNF2</t>
         </is>
       </c>
       <c r="D237" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי שמעון לביא באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/14?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי אלעזר בן עזריה באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/506?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E237" s="3" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F237" s="2" t="n">
-        <v>14</v>
+        <v>506</v>
       </c>
       <c r="G237" s="2" t="n"/>
     </row>
@@ -38849,24 +38849,24 @@
       </c>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>הרב נתן צבי פינקל (הסבא מסלבודקה)</t>
+          <t>רבי שמעון לביא</t>
         </is>
       </c>
       <c r="C238" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/4iRZ0WdzCGhxJrGTmkAzUf</t>
+          <t>https://open.spotify.com/episode/09sbxccxPcM8mqxUj6yDR4</t>
         </is>
       </c>
       <c r="D238" s="5" t="inlineStr">
         <is>
-          <t>📜 הרב נתן צבי פינקל (הסבא מסלבודקה) באוצר חכמים — המחקר המלא ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/324?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי שמעון לביא באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/14?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E238" s="3" t="n">
         <v>43</v>
       </c>
       <c r="F238" s="2" t="n">
-        <v>324</v>
+        <v>14</v>
       </c>
       <c r="G238" s="2" t="n"/>
     </row>
@@ -39686,24 +39686,24 @@
       </c>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>רבי יהושע בן חנניה</t>
+          <t>שרה אמנו</t>
         </is>
       </c>
       <c r="C269" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/4GuQl9XmYIYRZ48ooTWu4Q</t>
+          <t>https://open.spotify.com/episode/2XYXmPscJIo8gLmJov6AFc</t>
         </is>
       </c>
       <c r="D269" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי יהושע בן חנניה באוצר חכמים — המחקר המלא ורבותיו ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/503?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 שרה אמנו באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/448?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E269" s="3" t="n">
         <v>32</v>
       </c>
       <c r="F269" s="2" t="n">
-        <v>503</v>
+        <v>448</v>
       </c>
       <c r="G269" s="2" t="n"/>
     </row>
@@ -39713,24 +39713,24 @@
       </c>
       <c r="B270" s="4" t="inlineStr">
         <is>
-          <t>אדולף פראנק – הקבלה כפילוסופיה דתית</t>
+          <t>רבי יהושע בן חנניה</t>
         </is>
       </c>
       <c r="C270" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/5qiFDQTROpb7v21w4imqIE</t>
+          <t>https://open.spotify.com/episode/4GuQl9XmYIYRZ48ooTWu4Q</t>
         </is>
       </c>
       <c r="D270" s="5" t="inlineStr">
         <is>
-          <t>📜 אדולף פראנק באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/114?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי יהושע בן חנניה באוצר חכמים — המחקר המלא ורבותיו ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/503?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E270" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F270" s="2" t="n">
-        <v>114</v>
+        <v>503</v>
       </c>
       <c r="G270" s="2" t="n"/>
     </row>
@@ -39740,24 +39740,24 @@
       </c>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>הרב משה־צבי נריה – המהפכן הציוני־דתי שחי כל חייו בין חזון ל"בדיעבד" כעבודה: כשהעשייה היא דרך המלך</t>
+          <t>אדולף פראנק – הקבלה כפילוסופיה דתית</t>
         </is>
       </c>
       <c r="C271" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/43IiFgqfBCu9lLZIR07if7</t>
+          <t>https://open.spotify.com/episode/5qiFDQTROpb7v21w4imqIE</t>
         </is>
       </c>
       <c r="D271" s="5" t="inlineStr">
         <is>
-          <t>📜 הרב משה־צבי נריה באוצר חכמים — המחקר המלא ורבותיו ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/159?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 אדולף פראנק באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/114?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E271" s="3" t="n">
         <v>31</v>
       </c>
       <c r="F271" s="2" t="n">
-        <v>159</v>
+        <v>114</v>
       </c>
       <c r="G271" s="2" t="n"/>
     </row>
@@ -39767,24 +39767,24 @@
       </c>
       <c r="B272" s="4" t="inlineStr">
         <is>
-          <t>אסתר המלכה</t>
+          <t>הרב משה־צבי נריה – המהפכן הציוני־דתי שחי כל חייו בין חזון ל"בדיעבד" כעבודה: כשהעשייה היא דרך המלך</t>
         </is>
       </c>
       <c r="C272" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/4WssFuGXzvEgr2GstxIHfx</t>
+          <t>https://open.spotify.com/episode/43IiFgqfBCu9lLZIR07if7</t>
         </is>
       </c>
       <c r="D272" s="5" t="inlineStr">
         <is>
-          <t>📜 אסתר המלכה באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/268?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 הרב משה־צבי נריה באוצר חכמים — המחקר המלא ורבותיו ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/159?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E272" s="3" t="n">
         <v>31</v>
       </c>
       <c r="F272" s="2" t="n">
-        <v>268</v>
+        <v>159</v>
       </c>
       <c r="G272" s="2" t="n"/>
     </row>
@@ -39794,24 +39794,24 @@
       </c>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t>החיד״א (רבי חיים יוסף דוד אזולאי)</t>
+          <t>אסתר המלכה</t>
         </is>
       </c>
       <c r="C273" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/2MiUUx51sCblnVdS9i61Xq</t>
+          <t>https://open.spotify.com/episode/4WssFuGXzvEgr2GstxIHfx</t>
         </is>
       </c>
       <c r="D273" s="5" t="inlineStr">
         <is>
-          <t>📜 החיד״א (רבי חיים יוסף דוד אזולאי) באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/325?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 אסתר המלכה באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/268?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E273" s="3" t="n">
         <v>31</v>
       </c>
       <c r="F273" s="2" t="n">
-        <v>325</v>
+        <v>268</v>
       </c>
       <c r="G273" s="2" t="n"/>
     </row>
@@ -39821,24 +39821,24 @@
       </c>
       <c r="B274" s="4" t="inlineStr">
         <is>
-          <t>רבי מאיר בן שמעון המעילי</t>
+          <t>החיד״א (רבי חיים יוסף דוד אזולאי)</t>
         </is>
       </c>
       <c r="C274" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/2LqX1m0yUTIjrytoK1ZOD1</t>
+          <t>https://open.spotify.com/episode/2MiUUx51sCblnVdS9i61Xq</t>
         </is>
       </c>
       <c r="D274" s="5" t="inlineStr">
         <is>
-          <t>📜 רבי מאיר בן שמעון המעילי באוצר חכמים — המחקר המלא ורבותיו ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/393?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 החיד״א (רבי חיים יוסף דוד אזולאי) באוצר חכמים — המחקר המלא ורבותיו: https://ozar-chachamim-app.vercel.app/he/sage/325?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E274" s="3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F274" s="2" t="n">
-        <v>393</v>
+        <v>325</v>
       </c>
       <c r="G274" s="2" t="n"/>
     </row>
@@ -39848,24 +39848,24 @@
       </c>
       <c r="B275" s="4" t="inlineStr">
         <is>
-          <t>שרה אמנו</t>
+          <t>רבי מאיר בן שמעון המעילי</t>
         </is>
       </c>
       <c r="C275" s="6" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/episode/2XYXmPscJIo8gLmJov6AFc</t>
+          <t>https://open.spotify.com/episode/2LqX1m0yUTIjrytoK1ZOD1</t>
         </is>
       </c>
       <c r="D275" s="5" t="inlineStr">
         <is>
-          <t>📜 שרה אמנו באוצר חכמים — המחקר המלא: https://ozar-chachamim-app.vercel.app/he/sage/448?utm_source=spotify&amp;utm_medium=podcast</t>
+          <t>📜 רבי מאיר בן שמעון המעילי באוצר חכמים — המחקר המלא ורבותיו ותלמידיו: https://ozar-chachamim-app.vercel.app/he/sage/393?utm_source=spotify&amp;utm_medium=podcast</t>
         </is>
       </c>
       <c r="E275" s="3" t="n">
         <v>30</v>
       </c>
       <c r="F275" s="2" t="n">
-        <v>448</v>
+        <v>393</v>
       </c>
       <c r="G275" s="2" t="n"/>
     </row>
@@ -44047,7 +44047,7 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>נתוני הצפיות נלקחו מ־YouTube ב־2026-10-24.</t>
+          <t>נתוני הצפיות נלקחו מ־YouTube ב־2026-10-25.</t>
         </is>
       </c>
     </row>

</xml_diff>